<commit_message>
Massimo Dutti vendues 50 € sur Vinted : registres, stock et annonces à jour
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019NmjYPueKqR4wdTDtD4cw1
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Mode d'emploi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Livre des recettes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Registre des achats" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Objets mobiliers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livre des recettes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registre des achats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objets mobiliers" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Livre des recettes'!$A$5:$H$311</definedName>
@@ -11697,9 +11697,19 @@
           <t>Carte</t>
         </is>
       </c>
-      <c r="I22" s="11" t="inlineStr"/>
-      <c r="J22" s="12" t="inlineStr"/>
-      <c r="K22" s="11" t="inlineStr"/>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>Vendu sur Vinted, encaissement Vinted en attente</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="10">

</xml_diff>

<commit_message>
Vente des ballerines Massimo Dutti : registres, stock et procédure de vente
Livre des recettes (en attente d'encaissement Vinted), registre des objets
mobiliers et classeur de stock mis à jour. Procédure à chaque vente ajoutée
au roadmap et rappelée dans CLAUDE.md : retrait de Nouveautés et d'À la une.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vn9xBFDcKYi8h7FvBEWbRi
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Mode d'emploi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Livre des recettes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Registre des achats" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Objets mobiliers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livre des recettes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registre des achats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objets mobiliers" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Livre des recettes'!$A$5:$H$311</definedName>
@@ -121,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -145,6 +145,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1519,6 +1520,14 @@
       <c r="F12" s="11" t="n"/>
       <c r="G12" s="11" t="n"/>
       <c r="H12" s="11" t="n"/>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>Ballerines MASSIMO DUTTI P.40 — vendues le 19/10/2026 sur Vinted, facture n° 2026-002</t>
+        </is>
+      </c>
+      <c r="K12" s="19" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="10">
@@ -11697,9 +11706,19 @@
           <t>Carte</t>
         </is>
       </c>
-      <c r="I22" s="11" t="inlineStr"/>
-      <c r="J22" s="12" t="inlineStr"/>
-      <c r="K22" s="11" t="inlineStr"/>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>Vendue sur Vinted à Mme Ana Vidal Lorenzo (A Coruña, Espagne), facture n° 2026-002. Pointure à confirmer : 40 sur l'annonce, 41 sur la facture ADN.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="10">

</xml_diff>

<commit_message>
Facture 2026-002 sur une page, vente datée du 17/10/2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vn9xBFDcKYi8h7FvBEWbRi
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -1522,7 +1522,7 @@
       <c r="H12" s="11" t="n"/>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>Ballerines MASSIMO DUTTI P.40 — vendues le 19/10/2026 sur Vinted, facture n° 2026-002</t>
+          <t>Ballerines MASSIMO DUTTI P.40 — vendues le 17/10/2026 sur Vinted, facture n° 2026-002</t>
         </is>
       </c>
       <c r="K12" s="19" t="n">
@@ -11708,7 +11708,7 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>17/10/2026</t>
         </is>
       </c>
       <c r="J22" s="12" t="n">

</xml_diff>

<commit_message>
Renseigne le pseudonyme Vinted de l'acheteuse des ballerines Massimo Dutti (anavdlr)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>BALLERINES MASSIMO DUTTI P.41 — vendues le 17/10/2026 sur Vinted</t>
+          <t>BALLERINES MASSIMO DUTTI P.41 — vendues le 17/10/2026 sur Vinted à « anavdlr »</t>
         </is>
       </c>
       <c r="K9" s="13" t="n">
@@ -11795,7 +11795,7 @@
       </c>
       <c r="K22" s="11" t="inlineStr">
         <is>
-          <t>Vendu sur Vinted, encaissement en attente</t>
+          <t>Vendu sur Vinted à « anavdlr », encaissement en attente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Livre des recettes : colonne « Nature de la recette » et prestation de services du 3e trimestre (40 €)
Sépare l'achat-revente et la prestation de services dans les totaux et
dans le calcul de l'URSSAF (12,4 % / 21,3 %).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objets mobiliers" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Livre des recettes'!$A$5:$H$311</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Livre des recettes'!$A$5:$I$311</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Registre des achats'!$A$5:$G$350</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Objets mobiliers'!$A$5:$K$345</definedName>
   </definedNames>
@@ -1138,7 +1138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K311"/>
+  <dimension ref="A1:L311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1149,8 +1149,10 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1173,19 +1175,19 @@
           <t>On inscrit la vente le jour où l'argent arrive, pas le jour où elle est conclue. Ne jamais supprimer ni réordonner une ligne.</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>TOTAUX</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Recettes encaissées, total</t>
         </is>
       </c>
-      <c r="K4" s="6">
+      <c r="L4" s="6">
         <f>SUM(E6:E311)</f>
         <v/>
       </c>
@@ -1208,7 +1210,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Désignation de la vente</t>
+          <t>Désignation</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -1231,13 +1233,18 @@
           <t>Référence / pièce justificative</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>URSSAF à provisionner — 12,4 %</t>
-        </is>
-      </c>
-      <c r="K5" s="9">
-        <f>K4*0.124</f>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Nature de la recette</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  dont achat-revente</t>
+        </is>
+      </c>
+      <c r="L5" s="9">
+        <f>SUMIF(I6:I311,"Achat-revente",E6:E311)</f>
         <v/>
       </c>
     </row>
@@ -1279,13 +1286,18 @@
           <t>Facture n° 2026-001</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
-        <is>
-          <t>Reste après URSSAF</t>
-        </is>
-      </c>
-      <c r="K6" s="6">
-        <f>K4-K5</f>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>Achat-revente</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  dont prestations de services</t>
+        </is>
+      </c>
+      <c r="L6" s="9">
+        <f>SUMIF(I6:I311,"Prestation de services",E6:E311)</f>
         <v/>
       </c>
     </row>
@@ -1327,6 +1339,20 @@
           <t>Facture n° 2026-001</t>
         </is>
       </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Achat-revente</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>URSSAF — 12,4 % revente · 21,3 % prestations (taux à confirmer)</t>
+        </is>
+      </c>
+      <c r="L7" s="9">
+        <f>L5*0.124+L6*0.213</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10">
@@ -1366,10 +1392,19 @@
           <t>Facture n° 2026-001</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>EN ATTENTE D'ENCAISSEMENT</t>
-        </is>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>Achat-revente</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>Reste après URSSAF</t>
+        </is>
+      </c>
+      <c r="L8" s="9">
+        <f>L4-L7</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -1410,13 +1445,10 @@
           <t>Facture n° 2026-001</t>
         </is>
       </c>
-      <c r="J9" s="8" t="inlineStr">
-        <is>
-          <t>BALLERINES MASSIMO DUTTI P.41 — vendues le 17/10/2026 sur Vinted à « anavdlr »</t>
-        </is>
-      </c>
-      <c r="K9" s="13" t="n">
-        <v>50</v>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>Achat-revente</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1457,9 +1489,14 @@
           <t>Vinted — suivi Chronopost XU173687375JF, expédiée le 03/08/2026</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>Fonds retenus par Vinted. Relèvera du 4e trimestre 2026.</t>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>Achat-revente</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>EN ATTENTE D'ENCAISSEMENT</t>
         </is>
       </c>
     </row>
@@ -1501,10 +1538,18 @@
           <t>Achat : FB2026-5844 lot n°120</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>À BASCULER dans le registre le jour du virement, pas avant.</t>
-        </is>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Achat-revente</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>BALLERINES MASSIMO DUTTI P.41 — vendues le 17/10/2026 sur Vinted à « anavdlr »</t>
+        </is>
+      </c>
+      <c r="L11" s="13" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="12">
@@ -1545,6 +1590,16 @@
           <t>Vinted — vendue le 12/08/2026, expédiée le 14/08/2026 (Mondial Relay)</t>
         </is>
       </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>Achat-revente</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Fonds retenus par Vinted. Relèvera du 4e trimestre 2026.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="10">
@@ -1584,9 +1639,14 @@
           <t>Achat : FB2026-43716 lot n°199</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>DÉCLARATION URSSAF</t>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>Achat-revente</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>À BASCULER dans le registre le jour du virement, pas avant.</t>
         </is>
       </c>
     </row>
@@ -1628,9 +1688,9 @@
           <t>Achat : FB2026-5844 lot n°120</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>Le CA déclaré est le montant ENCAISSÉ sur la période, pas facturé.</t>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Achat-revente</t>
         </is>
       </c>
     </row>
@@ -1639,16 +1699,47 @@
         <f>IF(B15="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="12" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
-      <c r="H15" s="11" t="n"/>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Une vente d'août encaissée en septembre se déclare en septembre.</t>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>à compléter</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>à compléter</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Prestation de services commerciaux</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>à compléter</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>Déclarée au 3e trimestre 2026</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>Prestation de services</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>DÉCLARATION URSSAF</t>
         </is>
       </c>
     </row>
@@ -1664,9 +1755,10 @@
       <c r="F16" s="11" t="n"/>
       <c r="G16" s="11" t="n"/>
       <c r="H16" s="11" t="n"/>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>Filtrer la colonne « Date d'encaissement » pour isoler le trimestre.</t>
+      <c r="I16" s="11" t="n"/>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Le CA déclaré est le montant ENCAISSÉ sur la période, pas facturé.</t>
         </is>
       </c>
     </row>
@@ -1682,9 +1774,10 @@
       <c r="F17" s="11" t="n"/>
       <c r="G17" s="11" t="n"/>
       <c r="H17" s="11" t="n"/>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>Les 587 € encaissés relèvent du 3e trimestre 2026 — déclaration avant le 31 octobre.</t>
+      <c r="I17" s="11" t="n"/>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Une vente d'août encaissée en septembre se déclare en septembre.</t>
         </is>
       </c>
     </row>
@@ -1700,9 +1793,10 @@
       <c r="F18" s="11" t="n"/>
       <c r="G18" s="11" t="n"/>
       <c r="H18" s="11" t="n"/>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>Les 206,82 € d'apports personnels n'en font PAS partie : ce ne sont pas des recettes.</t>
+      <c r="I18" s="11" t="n"/>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Filtrer la colonne « Date d'encaissement » pour isoler le trimestre.</t>
         </is>
       </c>
     </row>
@@ -1718,9 +1812,10 @@
       <c r="F19" s="11" t="n"/>
       <c r="G19" s="11" t="n"/>
       <c r="H19" s="11" t="n"/>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>VENTES EN ESPÈCES — CE QU'IL FAUT GARDER</t>
+      <c r="I19" s="11" t="n"/>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>3e trimestre 2026 : 627 € déclarés (587 € de revente + 40 € de prestation), 81 € d'URSSAF payés.</t>
         </is>
       </c>
     </row>
@@ -1736,9 +1831,10 @@
       <c r="F20" s="11" t="n"/>
       <c r="G20" s="11" t="n"/>
       <c r="H20" s="11" t="n"/>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>Légal sans limite entre un professionnel et un particulier résidant en France jusqu'à 1 000 €</t>
+      <c r="I20" s="11" t="n"/>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>Les 206,82 € d'apports personnels n'en font PAS partie : ce ne sont pas des recettes.</t>
         </is>
       </c>
     </row>
@@ -1754,9 +1850,10 @@
       <c r="F21" s="11" t="n"/>
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="11" t="n"/>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>par transaction (art. L112-6 du code monétaire et financier). Toutes les ventes sont loin du seuil.</t>
+      <c r="I21" s="11" t="n"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>VENTES EN ESPÈCES — CE QU'IL FAUT GARDER</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1869,12 @@
       <c r="F22" s="11" t="n"/>
       <c r="G22" s="11" t="n"/>
       <c r="H22" s="11" t="n"/>
-      <c r="J22" s="5" t="inlineStr"/>
+      <c r="I22" s="11" t="n"/>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>Légal sans limite entre un professionnel et un particulier résidant en France jusqu'à 1 000 €</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="10">
@@ -1786,9 +1888,10 @@
       <c r="F23" s="11" t="n"/>
       <c r="G23" s="11" t="n"/>
       <c r="H23" s="11" t="n"/>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>La preuve d'une vente en espèces, c'est le registre plus le dépôt bancaire. Trois réflexes :</t>
+      <c r="I23" s="11" t="n"/>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>par transaction (art. L112-6 du code monétaire et financier). Toutes les ventes sont loin du seuil.</t>
         </is>
       </c>
     </row>
@@ -1804,11 +1907,8 @@
       <c r="F24" s="11" t="n"/>
       <c r="G24" s="11" t="n"/>
       <c r="H24" s="11" t="n"/>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1. Une note de vente par transaction — date, article, prix, nom de l'acheteur. Un carnet suffit.</t>
-        </is>
-      </c>
+      <c r="I24" s="11" t="n"/>
+      <c r="K24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="10">
@@ -1822,9 +1922,10 @@
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="11" t="n"/>
       <c r="H25" s="11" t="n"/>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2. Déposer sur le compte professionnel, pas sur le compte personnel : le détour brouille la piste.</t>
+      <c r="I25" s="11" t="n"/>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>La preuve d'une vente en espèces, c'est le registre plus le dépôt bancaire. Trois réflexes :</t>
         </is>
       </c>
     </row>
@@ -1840,13 +1941,11 @@
       <c r="F26" s="11" t="n"/>
       <c r="G26" s="11" t="n"/>
       <c r="H26" s="11" t="n"/>
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  3. Déposer par montants qui recoupent le registre, pour que le relevé confirme les lignes.</t>
-        </is>
-      </c>
-      <c r="K26" s="13" t="n">
-        <v>80</v>
+      <c r="I26" s="11" t="n"/>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. Une note de vente par transaction — date, article, prix, nom de l'acheteur. Un carnet suffit.</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -1861,13 +1960,11 @@
       <c r="F27" s="11" t="n"/>
       <c r="G27" s="11" t="n"/>
       <c r="H27" s="11" t="n"/>
-      <c r="J27" s="8" t="inlineStr">
-        <is>
-          <t>Baskets NIKE Air Max Moto 2K P.44.5 — gardées, 09/08/2026</t>
-        </is>
-      </c>
-      <c r="K27" s="13" t="n">
-        <v>70</v>
+      <c r="I27" s="11" t="n"/>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. Déposer sur le compte professionnel, pas sur le compte personnel : le détour brouille la piste.</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -1882,10 +1979,14 @@
       <c r="F28" s="11" t="n"/>
       <c r="G28" s="11" t="n"/>
       <c r="H28" s="11" t="n"/>
-      <c r="J28" s="8" t="inlineStr">
-        <is>
-          <t>Pompe ROBBY VP550W ligne 131 — gardée, 26/07/2026</t>
-        </is>
+      <c r="I28" s="11" t="n"/>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3. Déposer par montants qui recoupent le registre, pour que le relevé confirme les lignes.</t>
+        </is>
+      </c>
+      <c r="L28" s="13" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="29">
@@ -1900,10 +2001,14 @@
       <c r="F29" s="11" t="n"/>
       <c r="G29" s="11" t="n"/>
       <c r="H29" s="11" t="n"/>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>Booster High Class MEGA Dream ex M2a — gardé, 03/08/2026</t>
-        </is>
+      <c r="I29" s="11" t="n"/>
+      <c r="K29" s="8" t="inlineStr">
+        <is>
+          <t>Baskets NIKE Air Max Moto 2K P.44.5 — gardées, 09/08/2026</t>
+        </is>
+      </c>
+      <c r="L29" s="13" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="30">
@@ -1918,6 +2023,12 @@
       <c r="F30" s="11" t="n"/>
       <c r="G30" s="11" t="n"/>
       <c r="H30" s="11" t="n"/>
+      <c r="I30" s="11" t="n"/>
+      <c r="K30" s="8" t="inlineStr">
+        <is>
+          <t>Pompe ROBBY VP550W ligne 131 — gardée, 26/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="10">
@@ -1931,9 +2042,10 @@
       <c r="F31" s="11" t="n"/>
       <c r="G31" s="11" t="n"/>
       <c r="H31" s="11" t="n"/>
-      <c r="J31" s="5" t="inlineStr">
-        <is>
-          <t>Un micro-entrepreneur ne peut pas se vendre à lui-même : il n'y a pas deux personnes juridiques.</t>
+      <c r="I31" s="11" t="n"/>
+      <c r="K31" s="8" t="inlineStr">
+        <is>
+          <t>Booster High Class MEGA Dream ex M2a — gardé, 03/08/2026</t>
         </is>
       </c>
     </row>
@@ -1949,11 +2061,7 @@
       <c r="F32" s="11" t="n"/>
       <c r="G32" s="11" t="n"/>
       <c r="H32" s="11" t="n"/>
-      <c r="J32" s="5" t="inlineStr">
-        <is>
-          <t>Reprendre un article pour soi n'est pas une recette — aucun chiffre d'affaires, donc aucune URSSAF.</t>
-        </is>
-      </c>
+      <c r="I32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10">
@@ -1967,9 +2075,10 @@
       <c r="F33" s="11" t="n"/>
       <c r="G33" s="11" t="n"/>
       <c r="H33" s="11" t="n"/>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>Verser de l'argent de son compte personnel vers le compte pro est un APPORT, pas un encaissement.</t>
+      <c r="I33" s="11" t="n"/>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>Un micro-entrepreneur ne peut pas se vendre à lui-même : il n'y a pas deux personnes juridiques.</t>
         </is>
       </c>
     </row>
@@ -1985,9 +2094,10 @@
       <c r="F34" s="11" t="n"/>
       <c r="G34" s="11" t="n"/>
       <c r="H34" s="11" t="n"/>
-      <c r="J34" s="5" t="inlineStr">
-        <is>
-          <t>Ces lignes se notent en sortie au registre des objets mobiliers, jamais au livre des recettes.</t>
+      <c r="I34" s="11" t="n"/>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>Reprendre un article pour soi n'est pas une recette — aucun chiffre d'affaires, donc aucune URSSAF.</t>
         </is>
       </c>
     </row>
@@ -2003,6 +2113,12 @@
       <c r="F35" s="11" t="n"/>
       <c r="G35" s="11" t="n"/>
       <c r="H35" s="11" t="n"/>
+      <c r="I35" s="11" t="n"/>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>Verser de l'argent de son compte personnel vers le compte pro est un APPORT, pas un encaissement.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="10">
@@ -2016,6 +2132,12 @@
       <c r="F36" s="11" t="n"/>
       <c r="G36" s="11" t="n"/>
       <c r="H36" s="11" t="n"/>
+      <c r="I36" s="11" t="n"/>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>Ces lignes se notent en sortie au registre des objets mobiliers, jamais au livre des recettes.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="10">
@@ -2029,6 +2151,7 @@
       <c r="F37" s="11" t="n"/>
       <c r="G37" s="11" t="n"/>
       <c r="H37" s="11" t="n"/>
+      <c r="I37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10">
@@ -2042,6 +2165,7 @@
       <c r="F38" s="11" t="n"/>
       <c r="G38" s="11" t="n"/>
       <c r="H38" s="11" t="n"/>
+      <c r="I38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="10">
@@ -2055,6 +2179,7 @@
       <c r="F39" s="11" t="n"/>
       <c r="G39" s="11" t="n"/>
       <c r="H39" s="11" t="n"/>
+      <c r="I39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10">
@@ -2068,6 +2193,7 @@
       <c r="F40" s="11" t="n"/>
       <c r="G40" s="11" t="n"/>
       <c r="H40" s="11" t="n"/>
+      <c r="I40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10">
@@ -2081,6 +2207,7 @@
       <c r="F41" s="11" t="n"/>
       <c r="G41" s="11" t="n"/>
       <c r="H41" s="11" t="n"/>
+      <c r="I41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10">
@@ -2094,6 +2221,7 @@
       <c r="F42" s="11" t="n"/>
       <c r="G42" s="11" t="n"/>
       <c r="H42" s="11" t="n"/>
+      <c r="I42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="10">
@@ -2107,6 +2235,7 @@
       <c r="F43" s="11" t="n"/>
       <c r="G43" s="11" t="n"/>
       <c r="H43" s="11" t="n"/>
+      <c r="I43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="10">
@@ -2120,6 +2249,7 @@
       <c r="F44" s="11" t="n"/>
       <c r="G44" s="11" t="n"/>
       <c r="H44" s="11" t="n"/>
+      <c r="I44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="10">
@@ -2133,6 +2263,7 @@
       <c r="F45" s="11" t="n"/>
       <c r="G45" s="11" t="n"/>
       <c r="H45" s="11" t="n"/>
+      <c r="I45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10">
@@ -2146,6 +2277,7 @@
       <c r="F46" s="11" t="n"/>
       <c r="G46" s="11" t="n"/>
       <c r="H46" s="11" t="n"/>
+      <c r="I46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="10">
@@ -2159,6 +2291,7 @@
       <c r="F47" s="11" t="n"/>
       <c r="G47" s="11" t="n"/>
       <c r="H47" s="11" t="n"/>
+      <c r="I47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10">
@@ -2172,6 +2305,7 @@
       <c r="F48" s="11" t="n"/>
       <c r="G48" s="11" t="n"/>
       <c r="H48" s="11" t="n"/>
+      <c r="I48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="10">
@@ -2185,6 +2319,7 @@
       <c r="F49" s="11" t="n"/>
       <c r="G49" s="11" t="n"/>
       <c r="H49" s="11" t="n"/>
+      <c r="I49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="10">
@@ -2198,6 +2333,7 @@
       <c r="F50" s="11" t="n"/>
       <c r="G50" s="11" t="n"/>
       <c r="H50" s="11" t="n"/>
+      <c r="I50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="10">
@@ -2211,6 +2347,7 @@
       <c r="F51" s="11" t="n"/>
       <c r="G51" s="11" t="n"/>
       <c r="H51" s="11" t="n"/>
+      <c r="I51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10">
@@ -2224,6 +2361,7 @@
       <c r="F52" s="11" t="n"/>
       <c r="G52" s="11" t="n"/>
       <c r="H52" s="11" t="n"/>
+      <c r="I52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="10">
@@ -2237,6 +2375,7 @@
       <c r="F53" s="11" t="n"/>
       <c r="G53" s="11" t="n"/>
       <c r="H53" s="11" t="n"/>
+      <c r="I53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10">
@@ -2250,6 +2389,7 @@
       <c r="F54" s="11" t="n"/>
       <c r="G54" s="11" t="n"/>
       <c r="H54" s="11" t="n"/>
+      <c r="I54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="10">
@@ -2263,6 +2403,7 @@
       <c r="F55" s="11" t="n"/>
       <c r="G55" s="11" t="n"/>
       <c r="H55" s="11" t="n"/>
+      <c r="I55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10">
@@ -2276,6 +2417,7 @@
       <c r="F56" s="11" t="n"/>
       <c r="G56" s="11" t="n"/>
       <c r="H56" s="11" t="n"/>
+      <c r="I56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="10">
@@ -2289,6 +2431,7 @@
       <c r="F57" s="11" t="n"/>
       <c r="G57" s="11" t="n"/>
       <c r="H57" s="11" t="n"/>
+      <c r="I57" s="11" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10">
@@ -2302,6 +2445,7 @@
       <c r="F58" s="11" t="n"/>
       <c r="G58" s="11" t="n"/>
       <c r="H58" s="11" t="n"/>
+      <c r="I58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="10">
@@ -2315,6 +2459,7 @@
       <c r="F59" s="11" t="n"/>
       <c r="G59" s="11" t="n"/>
       <c r="H59" s="11" t="n"/>
+      <c r="I59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="10">
@@ -2328,6 +2473,7 @@
       <c r="F60" s="11" t="n"/>
       <c r="G60" s="11" t="n"/>
       <c r="H60" s="11" t="n"/>
+      <c r="I60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="10">
@@ -2341,6 +2487,7 @@
       <c r="F61" s="11" t="n"/>
       <c r="G61" s="11" t="n"/>
       <c r="H61" s="11" t="n"/>
+      <c r="I61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="10">
@@ -2354,6 +2501,7 @@
       <c r="F62" s="11" t="n"/>
       <c r="G62" s="11" t="n"/>
       <c r="H62" s="11" t="n"/>
+      <c r="I62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="10">
@@ -2367,6 +2515,7 @@
       <c r="F63" s="11" t="n"/>
       <c r="G63" s="11" t="n"/>
       <c r="H63" s="11" t="n"/>
+      <c r="I63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="10">
@@ -2380,6 +2529,7 @@
       <c r="F64" s="11" t="n"/>
       <c r="G64" s="11" t="n"/>
       <c r="H64" s="11" t="n"/>
+      <c r="I64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="10">
@@ -2393,6 +2543,7 @@
       <c r="F65" s="11" t="n"/>
       <c r="G65" s="11" t="n"/>
       <c r="H65" s="11" t="n"/>
+      <c r="I65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="10">
@@ -2406,6 +2557,7 @@
       <c r="F66" s="11" t="n"/>
       <c r="G66" s="11" t="n"/>
       <c r="H66" s="11" t="n"/>
+      <c r="I66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="10">
@@ -2419,6 +2571,7 @@
       <c r="F67" s="11" t="n"/>
       <c r="G67" s="11" t="n"/>
       <c r="H67" s="11" t="n"/>
+      <c r="I67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="10">
@@ -2432,6 +2585,7 @@
       <c r="F68" s="11" t="n"/>
       <c r="G68" s="11" t="n"/>
       <c r="H68" s="11" t="n"/>
+      <c r="I68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="10">
@@ -2445,6 +2599,7 @@
       <c r="F69" s="11" t="n"/>
       <c r="G69" s="11" t="n"/>
       <c r="H69" s="11" t="n"/>
+      <c r="I69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="10">
@@ -2458,6 +2613,7 @@
       <c r="F70" s="11" t="n"/>
       <c r="G70" s="11" t="n"/>
       <c r="H70" s="11" t="n"/>
+      <c r="I70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="10">
@@ -2471,6 +2627,7 @@
       <c r="F71" s="11" t="n"/>
       <c r="G71" s="11" t="n"/>
       <c r="H71" s="11" t="n"/>
+      <c r="I71" s="11" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="10">
@@ -2484,6 +2641,7 @@
       <c r="F72" s="11" t="n"/>
       <c r="G72" s="11" t="n"/>
       <c r="H72" s="11" t="n"/>
+      <c r="I72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="10">
@@ -2497,6 +2655,7 @@
       <c r="F73" s="11" t="n"/>
       <c r="G73" s="11" t="n"/>
       <c r="H73" s="11" t="n"/>
+      <c r="I73" s="11" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="10">
@@ -2510,6 +2669,7 @@
       <c r="F74" s="11" t="n"/>
       <c r="G74" s="11" t="n"/>
       <c r="H74" s="11" t="n"/>
+      <c r="I74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="10">
@@ -2523,6 +2683,7 @@
       <c r="F75" s="11" t="n"/>
       <c r="G75" s="11" t="n"/>
       <c r="H75" s="11" t="n"/>
+      <c r="I75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="10">
@@ -2536,6 +2697,7 @@
       <c r="F76" s="11" t="n"/>
       <c r="G76" s="11" t="n"/>
       <c r="H76" s="11" t="n"/>
+      <c r="I76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="10">
@@ -2549,6 +2711,7 @@
       <c r="F77" s="11" t="n"/>
       <c r="G77" s="11" t="n"/>
       <c r="H77" s="11" t="n"/>
+      <c r="I77" s="11" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="10">
@@ -2562,6 +2725,7 @@
       <c r="F78" s="11" t="n"/>
       <c r="G78" s="11" t="n"/>
       <c r="H78" s="11" t="n"/>
+      <c r="I78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="10">
@@ -2575,6 +2739,7 @@
       <c r="F79" s="11" t="n"/>
       <c r="G79" s="11" t="n"/>
       <c r="H79" s="11" t="n"/>
+      <c r="I79" s="11" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="10">
@@ -2588,6 +2753,7 @@
       <c r="F80" s="11" t="n"/>
       <c r="G80" s="11" t="n"/>
       <c r="H80" s="11" t="n"/>
+      <c r="I80" s="11" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="10">
@@ -2601,6 +2767,7 @@
       <c r="F81" s="11" t="n"/>
       <c r="G81" s="11" t="n"/>
       <c r="H81" s="11" t="n"/>
+      <c r="I81" s="11" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="10">
@@ -2614,6 +2781,7 @@
       <c r="F82" s="11" t="n"/>
       <c r="G82" s="11" t="n"/>
       <c r="H82" s="11" t="n"/>
+      <c r="I82" s="11" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="10">
@@ -2627,6 +2795,7 @@
       <c r="F83" s="11" t="n"/>
       <c r="G83" s="11" t="n"/>
       <c r="H83" s="11" t="n"/>
+      <c r="I83" s="11" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="10">
@@ -2640,6 +2809,7 @@
       <c r="F84" s="11" t="n"/>
       <c r="G84" s="11" t="n"/>
       <c r="H84" s="11" t="n"/>
+      <c r="I84" s="11" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="10">
@@ -2653,6 +2823,7 @@
       <c r="F85" s="11" t="n"/>
       <c r="G85" s="11" t="n"/>
       <c r="H85" s="11" t="n"/>
+      <c r="I85" s="11" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="10">
@@ -2666,6 +2837,7 @@
       <c r="F86" s="11" t="n"/>
       <c r="G86" s="11" t="n"/>
       <c r="H86" s="11" t="n"/>
+      <c r="I86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="10">
@@ -2679,6 +2851,7 @@
       <c r="F87" s="11" t="n"/>
       <c r="G87" s="11" t="n"/>
       <c r="H87" s="11" t="n"/>
+      <c r="I87" s="11" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="10">
@@ -2692,6 +2865,7 @@
       <c r="F88" s="11" t="n"/>
       <c r="G88" s="11" t="n"/>
       <c r="H88" s="11" t="n"/>
+      <c r="I88" s="11" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="10">
@@ -2705,6 +2879,7 @@
       <c r="F89" s="11" t="n"/>
       <c r="G89" s="11" t="n"/>
       <c r="H89" s="11" t="n"/>
+      <c r="I89" s="11" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="10">
@@ -2718,6 +2893,7 @@
       <c r="F90" s="11" t="n"/>
       <c r="G90" s="11" t="n"/>
       <c r="H90" s="11" t="n"/>
+      <c r="I90" s="11" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="10">
@@ -2731,6 +2907,7 @@
       <c r="F91" s="11" t="n"/>
       <c r="G91" s="11" t="n"/>
       <c r="H91" s="11" t="n"/>
+      <c r="I91" s="11" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="10">
@@ -2744,6 +2921,7 @@
       <c r="F92" s="11" t="n"/>
       <c r="G92" s="11" t="n"/>
       <c r="H92" s="11" t="n"/>
+      <c r="I92" s="11" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="10">
@@ -2757,6 +2935,7 @@
       <c r="F93" s="11" t="n"/>
       <c r="G93" s="11" t="n"/>
       <c r="H93" s="11" t="n"/>
+      <c r="I93" s="11" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="10">
@@ -2770,6 +2949,7 @@
       <c r="F94" s="11" t="n"/>
       <c r="G94" s="11" t="n"/>
       <c r="H94" s="11" t="n"/>
+      <c r="I94" s="11" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="10">
@@ -2783,6 +2963,7 @@
       <c r="F95" s="11" t="n"/>
       <c r="G95" s="11" t="n"/>
       <c r="H95" s="11" t="n"/>
+      <c r="I95" s="11" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="10">
@@ -2796,6 +2977,7 @@
       <c r="F96" s="11" t="n"/>
       <c r="G96" s="11" t="n"/>
       <c r="H96" s="11" t="n"/>
+      <c r="I96" s="11" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="10">
@@ -2809,6 +2991,7 @@
       <c r="F97" s="11" t="n"/>
       <c r="G97" s="11" t="n"/>
       <c r="H97" s="11" t="n"/>
+      <c r="I97" s="11" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="10">
@@ -2822,6 +3005,7 @@
       <c r="F98" s="11" t="n"/>
       <c r="G98" s="11" t="n"/>
       <c r="H98" s="11" t="n"/>
+      <c r="I98" s="11" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="10">
@@ -2835,6 +3019,7 @@
       <c r="F99" s="11" t="n"/>
       <c r="G99" s="11" t="n"/>
       <c r="H99" s="11" t="n"/>
+      <c r="I99" s="11" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="10">
@@ -2848,6 +3033,7 @@
       <c r="F100" s="11" t="n"/>
       <c r="G100" s="11" t="n"/>
       <c r="H100" s="11" t="n"/>
+      <c r="I100" s="11" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="10">
@@ -2861,6 +3047,7 @@
       <c r="F101" s="11" t="n"/>
       <c r="G101" s="11" t="n"/>
       <c r="H101" s="11" t="n"/>
+      <c r="I101" s="11" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="10">
@@ -2874,6 +3061,7 @@
       <c r="F102" s="11" t="n"/>
       <c r="G102" s="11" t="n"/>
       <c r="H102" s="11" t="n"/>
+      <c r="I102" s="11" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="10">
@@ -2887,6 +3075,7 @@
       <c r="F103" s="11" t="n"/>
       <c r="G103" s="11" t="n"/>
       <c r="H103" s="11" t="n"/>
+      <c r="I103" s="11" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="10">
@@ -2900,6 +3089,7 @@
       <c r="F104" s="11" t="n"/>
       <c r="G104" s="11" t="n"/>
       <c r="H104" s="11" t="n"/>
+      <c r="I104" s="11" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="10">
@@ -2913,6 +3103,7 @@
       <c r="F105" s="11" t="n"/>
       <c r="G105" s="11" t="n"/>
       <c r="H105" s="11" t="n"/>
+      <c r="I105" s="11" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="10">
@@ -2926,6 +3117,7 @@
       <c r="F106" s="11" t="n"/>
       <c r="G106" s="11" t="n"/>
       <c r="H106" s="11" t="n"/>
+      <c r="I106" s="11" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="10">
@@ -2939,6 +3131,7 @@
       <c r="F107" s="11" t="n"/>
       <c r="G107" s="11" t="n"/>
       <c r="H107" s="11" t="n"/>
+      <c r="I107" s="11" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="10">
@@ -2952,6 +3145,7 @@
       <c r="F108" s="11" t="n"/>
       <c r="G108" s="11" t="n"/>
       <c r="H108" s="11" t="n"/>
+      <c r="I108" s="11" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="10">
@@ -2965,6 +3159,7 @@
       <c r="F109" s="11" t="n"/>
       <c r="G109" s="11" t="n"/>
       <c r="H109" s="11" t="n"/>
+      <c r="I109" s="11" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="10">
@@ -2978,6 +3173,7 @@
       <c r="F110" s="11" t="n"/>
       <c r="G110" s="11" t="n"/>
       <c r="H110" s="11" t="n"/>
+      <c r="I110" s="11" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="10">
@@ -2991,6 +3187,7 @@
       <c r="F111" s="11" t="n"/>
       <c r="G111" s="11" t="n"/>
       <c r="H111" s="11" t="n"/>
+      <c r="I111" s="11" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="10">
@@ -3004,6 +3201,7 @@
       <c r="F112" s="11" t="n"/>
       <c r="G112" s="11" t="n"/>
       <c r="H112" s="11" t="n"/>
+      <c r="I112" s="11" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="10">
@@ -3017,6 +3215,7 @@
       <c r="F113" s="11" t="n"/>
       <c r="G113" s="11" t="n"/>
       <c r="H113" s="11" t="n"/>
+      <c r="I113" s="11" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="10">
@@ -3030,6 +3229,7 @@
       <c r="F114" s="11" t="n"/>
       <c r="G114" s="11" t="n"/>
       <c r="H114" s="11" t="n"/>
+      <c r="I114" s="11" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="10">
@@ -3043,6 +3243,7 @@
       <c r="F115" s="11" t="n"/>
       <c r="G115" s="11" t="n"/>
       <c r="H115" s="11" t="n"/>
+      <c r="I115" s="11" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="10">
@@ -3056,6 +3257,7 @@
       <c r="F116" s="11" t="n"/>
       <c r="G116" s="11" t="n"/>
       <c r="H116" s="11" t="n"/>
+      <c r="I116" s="11" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="10">
@@ -3069,6 +3271,7 @@
       <c r="F117" s="11" t="n"/>
       <c r="G117" s="11" t="n"/>
       <c r="H117" s="11" t="n"/>
+      <c r="I117" s="11" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="10">
@@ -3082,6 +3285,7 @@
       <c r="F118" s="11" t="n"/>
       <c r="G118" s="11" t="n"/>
       <c r="H118" s="11" t="n"/>
+      <c r="I118" s="11" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="10">
@@ -3095,6 +3299,7 @@
       <c r="F119" s="11" t="n"/>
       <c r="G119" s="11" t="n"/>
       <c r="H119" s="11" t="n"/>
+      <c r="I119" s="11" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="10">
@@ -3108,6 +3313,7 @@
       <c r="F120" s="11" t="n"/>
       <c r="G120" s="11" t="n"/>
       <c r="H120" s="11" t="n"/>
+      <c r="I120" s="11" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="10">
@@ -3121,6 +3327,7 @@
       <c r="F121" s="11" t="n"/>
       <c r="G121" s="11" t="n"/>
       <c r="H121" s="11" t="n"/>
+      <c r="I121" s="11" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="10">
@@ -3134,6 +3341,7 @@
       <c r="F122" s="11" t="n"/>
       <c r="G122" s="11" t="n"/>
       <c r="H122" s="11" t="n"/>
+      <c r="I122" s="11" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="10">
@@ -3147,6 +3355,7 @@
       <c r="F123" s="11" t="n"/>
       <c r="G123" s="11" t="n"/>
       <c r="H123" s="11" t="n"/>
+      <c r="I123" s="11" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="10">
@@ -3160,6 +3369,7 @@
       <c r="F124" s="11" t="n"/>
       <c r="G124" s="11" t="n"/>
       <c r="H124" s="11" t="n"/>
+      <c r="I124" s="11" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="10">
@@ -3173,6 +3383,7 @@
       <c r="F125" s="11" t="n"/>
       <c r="G125" s="11" t="n"/>
       <c r="H125" s="11" t="n"/>
+      <c r="I125" s="11" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="10">
@@ -3186,6 +3397,7 @@
       <c r="F126" s="11" t="n"/>
       <c r="G126" s="11" t="n"/>
       <c r="H126" s="11" t="n"/>
+      <c r="I126" s="11" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="10">
@@ -3199,6 +3411,7 @@
       <c r="F127" s="11" t="n"/>
       <c r="G127" s="11" t="n"/>
       <c r="H127" s="11" t="n"/>
+      <c r="I127" s="11" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="10">
@@ -3212,6 +3425,7 @@
       <c r="F128" s="11" t="n"/>
       <c r="G128" s="11" t="n"/>
       <c r="H128" s="11" t="n"/>
+      <c r="I128" s="11" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="10">
@@ -3225,6 +3439,7 @@
       <c r="F129" s="11" t="n"/>
       <c r="G129" s="11" t="n"/>
       <c r="H129" s="11" t="n"/>
+      <c r="I129" s="11" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="10">
@@ -3238,6 +3453,7 @@
       <c r="F130" s="11" t="n"/>
       <c r="G130" s="11" t="n"/>
       <c r="H130" s="11" t="n"/>
+      <c r="I130" s="11" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="10">
@@ -3251,6 +3467,7 @@
       <c r="F131" s="11" t="n"/>
       <c r="G131" s="11" t="n"/>
       <c r="H131" s="11" t="n"/>
+      <c r="I131" s="11" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="10">
@@ -3264,6 +3481,7 @@
       <c r="F132" s="11" t="n"/>
       <c r="G132" s="11" t="n"/>
       <c r="H132" s="11" t="n"/>
+      <c r="I132" s="11" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="10">
@@ -3277,6 +3495,7 @@
       <c r="F133" s="11" t="n"/>
       <c r="G133" s="11" t="n"/>
       <c r="H133" s="11" t="n"/>
+      <c r="I133" s="11" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="10">
@@ -3290,6 +3509,7 @@
       <c r="F134" s="11" t="n"/>
       <c r="G134" s="11" t="n"/>
       <c r="H134" s="11" t="n"/>
+      <c r="I134" s="11" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="10">
@@ -3303,6 +3523,7 @@
       <c r="F135" s="11" t="n"/>
       <c r="G135" s="11" t="n"/>
       <c r="H135" s="11" t="n"/>
+      <c r="I135" s="11" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="10">
@@ -3316,6 +3537,7 @@
       <c r="F136" s="11" t="n"/>
       <c r="G136" s="11" t="n"/>
       <c r="H136" s="11" t="n"/>
+      <c r="I136" s="11" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="10">
@@ -3329,6 +3551,7 @@
       <c r="F137" s="11" t="n"/>
       <c r="G137" s="11" t="n"/>
       <c r="H137" s="11" t="n"/>
+      <c r="I137" s="11" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="10">
@@ -3342,6 +3565,7 @@
       <c r="F138" s="11" t="n"/>
       <c r="G138" s="11" t="n"/>
       <c r="H138" s="11" t="n"/>
+      <c r="I138" s="11" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="10">
@@ -3355,6 +3579,7 @@
       <c r="F139" s="11" t="n"/>
       <c r="G139" s="11" t="n"/>
       <c r="H139" s="11" t="n"/>
+      <c r="I139" s="11" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="10">
@@ -3368,6 +3593,7 @@
       <c r="F140" s="11" t="n"/>
       <c r="G140" s="11" t="n"/>
       <c r="H140" s="11" t="n"/>
+      <c r="I140" s="11" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="10">
@@ -3381,6 +3607,7 @@
       <c r="F141" s="11" t="n"/>
       <c r="G141" s="11" t="n"/>
       <c r="H141" s="11" t="n"/>
+      <c r="I141" s="11" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="10">
@@ -3394,6 +3621,7 @@
       <c r="F142" s="11" t="n"/>
       <c r="G142" s="11" t="n"/>
       <c r="H142" s="11" t="n"/>
+      <c r="I142" s="11" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="10">
@@ -3407,6 +3635,7 @@
       <c r="F143" s="11" t="n"/>
       <c r="G143" s="11" t="n"/>
       <c r="H143" s="11" t="n"/>
+      <c r="I143" s="11" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="10">
@@ -3420,6 +3649,7 @@
       <c r="F144" s="11" t="n"/>
       <c r="G144" s="11" t="n"/>
       <c r="H144" s="11" t="n"/>
+      <c r="I144" s="11" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="10">
@@ -3433,6 +3663,7 @@
       <c r="F145" s="11" t="n"/>
       <c r="G145" s="11" t="n"/>
       <c r="H145" s="11" t="n"/>
+      <c r="I145" s="11" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="10">
@@ -3446,6 +3677,7 @@
       <c r="F146" s="11" t="n"/>
       <c r="G146" s="11" t="n"/>
       <c r="H146" s="11" t="n"/>
+      <c r="I146" s="11" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="10">
@@ -3459,6 +3691,7 @@
       <c r="F147" s="11" t="n"/>
       <c r="G147" s="11" t="n"/>
       <c r="H147" s="11" t="n"/>
+      <c r="I147" s="11" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="10">
@@ -3472,6 +3705,7 @@
       <c r="F148" s="11" t="n"/>
       <c r="G148" s="11" t="n"/>
       <c r="H148" s="11" t="n"/>
+      <c r="I148" s="11" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="10">
@@ -3485,6 +3719,7 @@
       <c r="F149" s="11" t="n"/>
       <c r="G149" s="11" t="n"/>
       <c r="H149" s="11" t="n"/>
+      <c r="I149" s="11" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="10">
@@ -3498,6 +3733,7 @@
       <c r="F150" s="11" t="n"/>
       <c r="G150" s="11" t="n"/>
       <c r="H150" s="11" t="n"/>
+      <c r="I150" s="11" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="10">
@@ -3511,6 +3747,7 @@
       <c r="F151" s="11" t="n"/>
       <c r="G151" s="11" t="n"/>
       <c r="H151" s="11" t="n"/>
+      <c r="I151" s="11" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="10">
@@ -3524,6 +3761,7 @@
       <c r="F152" s="11" t="n"/>
       <c r="G152" s="11" t="n"/>
       <c r="H152" s="11" t="n"/>
+      <c r="I152" s="11" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="10">
@@ -3537,6 +3775,7 @@
       <c r="F153" s="11" t="n"/>
       <c r="G153" s="11" t="n"/>
       <c r="H153" s="11" t="n"/>
+      <c r="I153" s="11" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="10">
@@ -3550,6 +3789,7 @@
       <c r="F154" s="11" t="n"/>
       <c r="G154" s="11" t="n"/>
       <c r="H154" s="11" t="n"/>
+      <c r="I154" s="11" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="10">
@@ -3563,6 +3803,7 @@
       <c r="F155" s="11" t="n"/>
       <c r="G155" s="11" t="n"/>
       <c r="H155" s="11" t="n"/>
+      <c r="I155" s="11" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="10">
@@ -3576,6 +3817,7 @@
       <c r="F156" s="11" t="n"/>
       <c r="G156" s="11" t="n"/>
       <c r="H156" s="11" t="n"/>
+      <c r="I156" s="11" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="10">
@@ -3589,6 +3831,7 @@
       <c r="F157" s="11" t="n"/>
       <c r="G157" s="11" t="n"/>
       <c r="H157" s="11" t="n"/>
+      <c r="I157" s="11" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="10">
@@ -3602,6 +3845,7 @@
       <c r="F158" s="11" t="n"/>
       <c r="G158" s="11" t="n"/>
       <c r="H158" s="11" t="n"/>
+      <c r="I158" s="11" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="10">
@@ -3615,6 +3859,7 @@
       <c r="F159" s="11" t="n"/>
       <c r="G159" s="11" t="n"/>
       <c r="H159" s="11" t="n"/>
+      <c r="I159" s="11" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="10">
@@ -3628,6 +3873,7 @@
       <c r="F160" s="11" t="n"/>
       <c r="G160" s="11" t="n"/>
       <c r="H160" s="11" t="n"/>
+      <c r="I160" s="11" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="10">
@@ -3641,6 +3887,7 @@
       <c r="F161" s="11" t="n"/>
       <c r="G161" s="11" t="n"/>
       <c r="H161" s="11" t="n"/>
+      <c r="I161" s="11" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="10">
@@ -3654,6 +3901,7 @@
       <c r="F162" s="11" t="n"/>
       <c r="G162" s="11" t="n"/>
       <c r="H162" s="11" t="n"/>
+      <c r="I162" s="11" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="10">
@@ -3667,6 +3915,7 @@
       <c r="F163" s="11" t="n"/>
       <c r="G163" s="11" t="n"/>
       <c r="H163" s="11" t="n"/>
+      <c r="I163" s="11" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="10">
@@ -3680,6 +3929,7 @@
       <c r="F164" s="11" t="n"/>
       <c r="G164" s="11" t="n"/>
       <c r="H164" s="11" t="n"/>
+      <c r="I164" s="11" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="10">
@@ -3693,6 +3943,7 @@
       <c r="F165" s="11" t="n"/>
       <c r="G165" s="11" t="n"/>
       <c r="H165" s="11" t="n"/>
+      <c r="I165" s="11" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="10">
@@ -3706,6 +3957,7 @@
       <c r="F166" s="11" t="n"/>
       <c r="G166" s="11" t="n"/>
       <c r="H166" s="11" t="n"/>
+      <c r="I166" s="11" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="10">
@@ -3719,6 +3971,7 @@
       <c r="F167" s="11" t="n"/>
       <c r="G167" s="11" t="n"/>
       <c r="H167" s="11" t="n"/>
+      <c r="I167" s="11" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="10">
@@ -3732,6 +3985,7 @@
       <c r="F168" s="11" t="n"/>
       <c r="G168" s="11" t="n"/>
       <c r="H168" s="11" t="n"/>
+      <c r="I168" s="11" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="10">
@@ -3745,6 +3999,7 @@
       <c r="F169" s="11" t="n"/>
       <c r="G169" s="11" t="n"/>
       <c r="H169" s="11" t="n"/>
+      <c r="I169" s="11" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="10">
@@ -3758,6 +4013,7 @@
       <c r="F170" s="11" t="n"/>
       <c r="G170" s="11" t="n"/>
       <c r="H170" s="11" t="n"/>
+      <c r="I170" s="11" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="10">
@@ -3771,6 +4027,7 @@
       <c r="F171" s="11" t="n"/>
       <c r="G171" s="11" t="n"/>
       <c r="H171" s="11" t="n"/>
+      <c r="I171" s="11" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="10">
@@ -3784,6 +4041,7 @@
       <c r="F172" s="11" t="n"/>
       <c r="G172" s="11" t="n"/>
       <c r="H172" s="11" t="n"/>
+      <c r="I172" s="11" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="10">
@@ -3797,6 +4055,7 @@
       <c r="F173" s="11" t="n"/>
       <c r="G173" s="11" t="n"/>
       <c r="H173" s="11" t="n"/>
+      <c r="I173" s="11" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="10">
@@ -3810,6 +4069,7 @@
       <c r="F174" s="11" t="n"/>
       <c r="G174" s="11" t="n"/>
       <c r="H174" s="11" t="n"/>
+      <c r="I174" s="11" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="10">
@@ -3823,6 +4083,7 @@
       <c r="F175" s="11" t="n"/>
       <c r="G175" s="11" t="n"/>
       <c r="H175" s="11" t="n"/>
+      <c r="I175" s="11" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="10">
@@ -3836,6 +4097,7 @@
       <c r="F176" s="11" t="n"/>
       <c r="G176" s="11" t="n"/>
       <c r="H176" s="11" t="n"/>
+      <c r="I176" s="11" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="10">
@@ -3849,6 +4111,7 @@
       <c r="F177" s="11" t="n"/>
       <c r="G177" s="11" t="n"/>
       <c r="H177" s="11" t="n"/>
+      <c r="I177" s="11" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="10">
@@ -3862,6 +4125,7 @@
       <c r="F178" s="11" t="n"/>
       <c r="G178" s="11" t="n"/>
       <c r="H178" s="11" t="n"/>
+      <c r="I178" s="11" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="10">
@@ -3875,6 +4139,7 @@
       <c r="F179" s="11" t="n"/>
       <c r="G179" s="11" t="n"/>
       <c r="H179" s="11" t="n"/>
+      <c r="I179" s="11" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="10">
@@ -3888,6 +4153,7 @@
       <c r="F180" s="11" t="n"/>
       <c r="G180" s="11" t="n"/>
       <c r="H180" s="11" t="n"/>
+      <c r="I180" s="11" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="10">
@@ -3901,6 +4167,7 @@
       <c r="F181" s="11" t="n"/>
       <c r="G181" s="11" t="n"/>
       <c r="H181" s="11" t="n"/>
+      <c r="I181" s="11" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="10">
@@ -3914,6 +4181,7 @@
       <c r="F182" s="11" t="n"/>
       <c r="G182" s="11" t="n"/>
       <c r="H182" s="11" t="n"/>
+      <c r="I182" s="11" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="10">
@@ -3927,6 +4195,7 @@
       <c r="F183" s="11" t="n"/>
       <c r="G183" s="11" t="n"/>
       <c r="H183" s="11" t="n"/>
+      <c r="I183" s="11" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="10">
@@ -3940,6 +4209,7 @@
       <c r="F184" s="11" t="n"/>
       <c r="G184" s="11" t="n"/>
       <c r="H184" s="11" t="n"/>
+      <c r="I184" s="11" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="10">
@@ -3953,6 +4223,7 @@
       <c r="F185" s="11" t="n"/>
       <c r="G185" s="11" t="n"/>
       <c r="H185" s="11" t="n"/>
+      <c r="I185" s="11" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="10">
@@ -3966,6 +4237,7 @@
       <c r="F186" s="11" t="n"/>
       <c r="G186" s="11" t="n"/>
       <c r="H186" s="11" t="n"/>
+      <c r="I186" s="11" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="10">
@@ -3979,6 +4251,7 @@
       <c r="F187" s="11" t="n"/>
       <c r="G187" s="11" t="n"/>
       <c r="H187" s="11" t="n"/>
+      <c r="I187" s="11" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="10">
@@ -3992,6 +4265,7 @@
       <c r="F188" s="11" t="n"/>
       <c r="G188" s="11" t="n"/>
       <c r="H188" s="11" t="n"/>
+      <c r="I188" s="11" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="10">
@@ -4005,6 +4279,7 @@
       <c r="F189" s="11" t="n"/>
       <c r="G189" s="11" t="n"/>
       <c r="H189" s="11" t="n"/>
+      <c r="I189" s="11" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="10">
@@ -4018,6 +4293,7 @@
       <c r="F190" s="11" t="n"/>
       <c r="G190" s="11" t="n"/>
       <c r="H190" s="11" t="n"/>
+      <c r="I190" s="11" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="10">
@@ -4031,6 +4307,7 @@
       <c r="F191" s="11" t="n"/>
       <c r="G191" s="11" t="n"/>
       <c r="H191" s="11" t="n"/>
+      <c r="I191" s="11" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="10">
@@ -4044,6 +4321,7 @@
       <c r="F192" s="11" t="n"/>
       <c r="G192" s="11" t="n"/>
       <c r="H192" s="11" t="n"/>
+      <c r="I192" s="11" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="10">
@@ -4057,6 +4335,7 @@
       <c r="F193" s="11" t="n"/>
       <c r="G193" s="11" t="n"/>
       <c r="H193" s="11" t="n"/>
+      <c r="I193" s="11" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="10">
@@ -4070,6 +4349,7 @@
       <c r="F194" s="11" t="n"/>
       <c r="G194" s="11" t="n"/>
       <c r="H194" s="11" t="n"/>
+      <c r="I194" s="11" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="10">
@@ -4083,6 +4363,7 @@
       <c r="F195" s="11" t="n"/>
       <c r="G195" s="11" t="n"/>
       <c r="H195" s="11" t="n"/>
+      <c r="I195" s="11" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="10">
@@ -4096,6 +4377,7 @@
       <c r="F196" s="11" t="n"/>
       <c r="G196" s="11" t="n"/>
       <c r="H196" s="11" t="n"/>
+      <c r="I196" s="11" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="10">
@@ -4109,6 +4391,7 @@
       <c r="F197" s="11" t="n"/>
       <c r="G197" s="11" t="n"/>
       <c r="H197" s="11" t="n"/>
+      <c r="I197" s="11" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="10">
@@ -4122,6 +4405,7 @@
       <c r="F198" s="11" t="n"/>
       <c r="G198" s="11" t="n"/>
       <c r="H198" s="11" t="n"/>
+      <c r="I198" s="11" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="10">
@@ -4135,6 +4419,7 @@
       <c r="F199" s="11" t="n"/>
       <c r="G199" s="11" t="n"/>
       <c r="H199" s="11" t="n"/>
+      <c r="I199" s="11" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="10">
@@ -4148,6 +4433,7 @@
       <c r="F200" s="11" t="n"/>
       <c r="G200" s="11" t="n"/>
       <c r="H200" s="11" t="n"/>
+      <c r="I200" s="11" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="10">
@@ -4161,6 +4447,7 @@
       <c r="F201" s="11" t="n"/>
       <c r="G201" s="11" t="n"/>
       <c r="H201" s="11" t="n"/>
+      <c r="I201" s="11" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="10">
@@ -4174,6 +4461,7 @@
       <c r="F202" s="11" t="n"/>
       <c r="G202" s="11" t="n"/>
       <c r="H202" s="11" t="n"/>
+      <c r="I202" s="11" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="10">
@@ -4187,6 +4475,7 @@
       <c r="F203" s="11" t="n"/>
       <c r="G203" s="11" t="n"/>
       <c r="H203" s="11" t="n"/>
+      <c r="I203" s="11" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="10">
@@ -4200,6 +4489,7 @@
       <c r="F204" s="11" t="n"/>
       <c r="G204" s="11" t="n"/>
       <c r="H204" s="11" t="n"/>
+      <c r="I204" s="11" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="10">
@@ -4213,6 +4503,7 @@
       <c r="F205" s="11" t="n"/>
       <c r="G205" s="11" t="n"/>
       <c r="H205" s="11" t="n"/>
+      <c r="I205" s="11" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="10">
@@ -4226,6 +4517,7 @@
       <c r="F206" s="11" t="n"/>
       <c r="G206" s="11" t="n"/>
       <c r="H206" s="11" t="n"/>
+      <c r="I206" s="11" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="10">
@@ -4239,6 +4531,7 @@
       <c r="F207" s="11" t="n"/>
       <c r="G207" s="11" t="n"/>
       <c r="H207" s="11" t="n"/>
+      <c r="I207" s="11" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="10">
@@ -4252,6 +4545,7 @@
       <c r="F208" s="11" t="n"/>
       <c r="G208" s="11" t="n"/>
       <c r="H208" s="11" t="n"/>
+      <c r="I208" s="11" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="10">
@@ -4265,6 +4559,7 @@
       <c r="F209" s="11" t="n"/>
       <c r="G209" s="11" t="n"/>
       <c r="H209" s="11" t="n"/>
+      <c r="I209" s="11" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="10">
@@ -4278,6 +4573,7 @@
       <c r="F210" s="11" t="n"/>
       <c r="G210" s="11" t="n"/>
       <c r="H210" s="11" t="n"/>
+      <c r="I210" s="11" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="10">
@@ -4291,6 +4587,7 @@
       <c r="F211" s="11" t="n"/>
       <c r="G211" s="11" t="n"/>
       <c r="H211" s="11" t="n"/>
+      <c r="I211" s="11" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="10">
@@ -4304,6 +4601,7 @@
       <c r="F212" s="11" t="n"/>
       <c r="G212" s="11" t="n"/>
       <c r="H212" s="11" t="n"/>
+      <c r="I212" s="11" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="10">
@@ -4317,6 +4615,7 @@
       <c r="F213" s="11" t="n"/>
       <c r="G213" s="11" t="n"/>
       <c r="H213" s="11" t="n"/>
+      <c r="I213" s="11" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="10">
@@ -4330,6 +4629,7 @@
       <c r="F214" s="11" t="n"/>
       <c r="G214" s="11" t="n"/>
       <c r="H214" s="11" t="n"/>
+      <c r="I214" s="11" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="10">
@@ -4343,6 +4643,7 @@
       <c r="F215" s="11" t="n"/>
       <c r="G215" s="11" t="n"/>
       <c r="H215" s="11" t="n"/>
+      <c r="I215" s="11" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="10">
@@ -4356,6 +4657,7 @@
       <c r="F216" s="11" t="n"/>
       <c r="G216" s="11" t="n"/>
       <c r="H216" s="11" t="n"/>
+      <c r="I216" s="11" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="10">
@@ -4369,6 +4671,7 @@
       <c r="F217" s="11" t="n"/>
       <c r="G217" s="11" t="n"/>
       <c r="H217" s="11" t="n"/>
+      <c r="I217" s="11" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="10">
@@ -4382,6 +4685,7 @@
       <c r="F218" s="11" t="n"/>
       <c r="G218" s="11" t="n"/>
       <c r="H218" s="11" t="n"/>
+      <c r="I218" s="11" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="10">
@@ -4395,6 +4699,7 @@
       <c r="F219" s="11" t="n"/>
       <c r="G219" s="11" t="n"/>
       <c r="H219" s="11" t="n"/>
+      <c r="I219" s="11" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="10">
@@ -4408,6 +4713,7 @@
       <c r="F220" s="11" t="n"/>
       <c r="G220" s="11" t="n"/>
       <c r="H220" s="11" t="n"/>
+      <c r="I220" s="11" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="10">
@@ -4421,6 +4727,7 @@
       <c r="F221" s="11" t="n"/>
       <c r="G221" s="11" t="n"/>
       <c r="H221" s="11" t="n"/>
+      <c r="I221" s="11" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="10">
@@ -4434,6 +4741,7 @@
       <c r="F222" s="11" t="n"/>
       <c r="G222" s="11" t="n"/>
       <c r="H222" s="11" t="n"/>
+      <c r="I222" s="11" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="10">
@@ -4447,6 +4755,7 @@
       <c r="F223" s="11" t="n"/>
       <c r="G223" s="11" t="n"/>
       <c r="H223" s="11" t="n"/>
+      <c r="I223" s="11" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="10">
@@ -4460,6 +4769,7 @@
       <c r="F224" s="11" t="n"/>
       <c r="G224" s="11" t="n"/>
       <c r="H224" s="11" t="n"/>
+      <c r="I224" s="11" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="10">
@@ -4473,6 +4783,7 @@
       <c r="F225" s="11" t="n"/>
       <c r="G225" s="11" t="n"/>
       <c r="H225" s="11" t="n"/>
+      <c r="I225" s="11" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="10">
@@ -4486,6 +4797,7 @@
       <c r="F226" s="11" t="n"/>
       <c r="G226" s="11" t="n"/>
       <c r="H226" s="11" t="n"/>
+      <c r="I226" s="11" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="10">
@@ -4499,6 +4811,7 @@
       <c r="F227" s="11" t="n"/>
       <c r="G227" s="11" t="n"/>
       <c r="H227" s="11" t="n"/>
+      <c r="I227" s="11" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="10">
@@ -4512,6 +4825,7 @@
       <c r="F228" s="11" t="n"/>
       <c r="G228" s="11" t="n"/>
       <c r="H228" s="11" t="n"/>
+      <c r="I228" s="11" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="10">
@@ -4525,6 +4839,7 @@
       <c r="F229" s="11" t="n"/>
       <c r="G229" s="11" t="n"/>
       <c r="H229" s="11" t="n"/>
+      <c r="I229" s="11" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="10">
@@ -4538,6 +4853,7 @@
       <c r="F230" s="11" t="n"/>
       <c r="G230" s="11" t="n"/>
       <c r="H230" s="11" t="n"/>
+      <c r="I230" s="11" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="10">
@@ -4551,6 +4867,7 @@
       <c r="F231" s="11" t="n"/>
       <c r="G231" s="11" t="n"/>
       <c r="H231" s="11" t="n"/>
+      <c r="I231" s="11" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="10">
@@ -4564,6 +4881,7 @@
       <c r="F232" s="11" t="n"/>
       <c r="G232" s="11" t="n"/>
       <c r="H232" s="11" t="n"/>
+      <c r="I232" s="11" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="10">
@@ -4577,6 +4895,7 @@
       <c r="F233" s="11" t="n"/>
       <c r="G233" s="11" t="n"/>
       <c r="H233" s="11" t="n"/>
+      <c r="I233" s="11" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="10">
@@ -4590,6 +4909,7 @@
       <c r="F234" s="11" t="n"/>
       <c r="G234" s="11" t="n"/>
       <c r="H234" s="11" t="n"/>
+      <c r="I234" s="11" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="10">
@@ -4603,6 +4923,7 @@
       <c r="F235" s="11" t="n"/>
       <c r="G235" s="11" t="n"/>
       <c r="H235" s="11" t="n"/>
+      <c r="I235" s="11" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="10">
@@ -4616,6 +4937,7 @@
       <c r="F236" s="11" t="n"/>
       <c r="G236" s="11" t="n"/>
       <c r="H236" s="11" t="n"/>
+      <c r="I236" s="11" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="10">
@@ -4629,6 +4951,7 @@
       <c r="F237" s="11" t="n"/>
       <c r="G237" s="11" t="n"/>
       <c r="H237" s="11" t="n"/>
+      <c r="I237" s="11" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="10">
@@ -4642,6 +4965,7 @@
       <c r="F238" s="11" t="n"/>
       <c r="G238" s="11" t="n"/>
       <c r="H238" s="11" t="n"/>
+      <c r="I238" s="11" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="10">
@@ -4655,6 +4979,7 @@
       <c r="F239" s="11" t="n"/>
       <c r="G239" s="11" t="n"/>
       <c r="H239" s="11" t="n"/>
+      <c r="I239" s="11" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="10">
@@ -4668,6 +4993,7 @@
       <c r="F240" s="11" t="n"/>
       <c r="G240" s="11" t="n"/>
       <c r="H240" s="11" t="n"/>
+      <c r="I240" s="11" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="10">
@@ -4681,6 +5007,7 @@
       <c r="F241" s="11" t="n"/>
       <c r="G241" s="11" t="n"/>
       <c r="H241" s="11" t="n"/>
+      <c r="I241" s="11" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="10">
@@ -4694,6 +5021,7 @@
       <c r="F242" s="11" t="n"/>
       <c r="G242" s="11" t="n"/>
       <c r="H242" s="11" t="n"/>
+      <c r="I242" s="11" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="10">
@@ -4707,6 +5035,7 @@
       <c r="F243" s="11" t="n"/>
       <c r="G243" s="11" t="n"/>
       <c r="H243" s="11" t="n"/>
+      <c r="I243" s="11" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="10">
@@ -4720,6 +5049,7 @@
       <c r="F244" s="11" t="n"/>
       <c r="G244" s="11" t="n"/>
       <c r="H244" s="11" t="n"/>
+      <c r="I244" s="11" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="10">
@@ -4733,6 +5063,7 @@
       <c r="F245" s="11" t="n"/>
       <c r="G245" s="11" t="n"/>
       <c r="H245" s="11" t="n"/>
+      <c r="I245" s="11" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="10">
@@ -4746,6 +5077,7 @@
       <c r="F246" s="11" t="n"/>
       <c r="G246" s="11" t="n"/>
       <c r="H246" s="11" t="n"/>
+      <c r="I246" s="11" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="10">
@@ -4759,6 +5091,7 @@
       <c r="F247" s="11" t="n"/>
       <c r="G247" s="11" t="n"/>
       <c r="H247" s="11" t="n"/>
+      <c r="I247" s="11" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="10">
@@ -4772,6 +5105,7 @@
       <c r="F248" s="11" t="n"/>
       <c r="G248" s="11" t="n"/>
       <c r="H248" s="11" t="n"/>
+      <c r="I248" s="11" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="10">
@@ -4785,6 +5119,7 @@
       <c r="F249" s="11" t="n"/>
       <c r="G249" s="11" t="n"/>
       <c r="H249" s="11" t="n"/>
+      <c r="I249" s="11" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="10">
@@ -4798,6 +5133,7 @@
       <c r="F250" s="11" t="n"/>
       <c r="G250" s="11" t="n"/>
       <c r="H250" s="11" t="n"/>
+      <c r="I250" s="11" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="10">
@@ -4811,6 +5147,7 @@
       <c r="F251" s="11" t="n"/>
       <c r="G251" s="11" t="n"/>
       <c r="H251" s="11" t="n"/>
+      <c r="I251" s="11" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="10">
@@ -4824,6 +5161,7 @@
       <c r="F252" s="11" t="n"/>
       <c r="G252" s="11" t="n"/>
       <c r="H252" s="11" t="n"/>
+      <c r="I252" s="11" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="10">
@@ -4837,6 +5175,7 @@
       <c r="F253" s="11" t="n"/>
       <c r="G253" s="11" t="n"/>
       <c r="H253" s="11" t="n"/>
+      <c r="I253" s="11" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="10">
@@ -4850,6 +5189,7 @@
       <c r="F254" s="11" t="n"/>
       <c r="G254" s="11" t="n"/>
       <c r="H254" s="11" t="n"/>
+      <c r="I254" s="11" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="10">
@@ -4863,6 +5203,7 @@
       <c r="F255" s="11" t="n"/>
       <c r="G255" s="11" t="n"/>
       <c r="H255" s="11" t="n"/>
+      <c r="I255" s="11" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="10">
@@ -4876,6 +5217,7 @@
       <c r="F256" s="11" t="n"/>
       <c r="G256" s="11" t="n"/>
       <c r="H256" s="11" t="n"/>
+      <c r="I256" s="11" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="10">
@@ -4889,6 +5231,7 @@
       <c r="F257" s="11" t="n"/>
       <c r="G257" s="11" t="n"/>
       <c r="H257" s="11" t="n"/>
+      <c r="I257" s="11" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="10">
@@ -4902,6 +5245,7 @@
       <c r="F258" s="11" t="n"/>
       <c r="G258" s="11" t="n"/>
       <c r="H258" s="11" t="n"/>
+      <c r="I258" s="11" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="10">
@@ -4915,6 +5259,7 @@
       <c r="F259" s="11" t="n"/>
       <c r="G259" s="11" t="n"/>
       <c r="H259" s="11" t="n"/>
+      <c r="I259" s="11" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="10">
@@ -4928,6 +5273,7 @@
       <c r="F260" s="11" t="n"/>
       <c r="G260" s="11" t="n"/>
       <c r="H260" s="11" t="n"/>
+      <c r="I260" s="11" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="10">
@@ -4941,6 +5287,7 @@
       <c r="F261" s="11" t="n"/>
       <c r="G261" s="11" t="n"/>
       <c r="H261" s="11" t="n"/>
+      <c r="I261" s="11" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="10">
@@ -4954,6 +5301,7 @@
       <c r="F262" s="11" t="n"/>
       <c r="G262" s="11" t="n"/>
       <c r="H262" s="11" t="n"/>
+      <c r="I262" s="11" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="10">
@@ -4967,6 +5315,7 @@
       <c r="F263" s="11" t="n"/>
       <c r="G263" s="11" t="n"/>
       <c r="H263" s="11" t="n"/>
+      <c r="I263" s="11" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="10">
@@ -4980,6 +5329,7 @@
       <c r="F264" s="11" t="n"/>
       <c r="G264" s="11" t="n"/>
       <c r="H264" s="11" t="n"/>
+      <c r="I264" s="11" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="10">
@@ -4993,6 +5343,7 @@
       <c r="F265" s="11" t="n"/>
       <c r="G265" s="11" t="n"/>
       <c r="H265" s="11" t="n"/>
+      <c r="I265" s="11" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="10">
@@ -5006,6 +5357,7 @@
       <c r="F266" s="11" t="n"/>
       <c r="G266" s="11" t="n"/>
       <c r="H266" s="11" t="n"/>
+      <c r="I266" s="11" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="10">
@@ -5019,6 +5371,7 @@
       <c r="F267" s="11" t="n"/>
       <c r="G267" s="11" t="n"/>
       <c r="H267" s="11" t="n"/>
+      <c r="I267" s="11" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="10">
@@ -5032,6 +5385,7 @@
       <c r="F268" s="11" t="n"/>
       <c r="G268" s="11" t="n"/>
       <c r="H268" s="11" t="n"/>
+      <c r="I268" s="11" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="10">
@@ -5045,6 +5399,7 @@
       <c r="F269" s="11" t="n"/>
       <c r="G269" s="11" t="n"/>
       <c r="H269" s="11" t="n"/>
+      <c r="I269" s="11" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="10">
@@ -5058,6 +5413,7 @@
       <c r="F270" s="11" t="n"/>
       <c r="G270" s="11" t="n"/>
       <c r="H270" s="11" t="n"/>
+      <c r="I270" s="11" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="10">
@@ -5071,6 +5427,7 @@
       <c r="F271" s="11" t="n"/>
       <c r="G271" s="11" t="n"/>
       <c r="H271" s="11" t="n"/>
+      <c r="I271" s="11" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="10">
@@ -5084,6 +5441,7 @@
       <c r="F272" s="11" t="n"/>
       <c r="G272" s="11" t="n"/>
       <c r="H272" s="11" t="n"/>
+      <c r="I272" s="11" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="10">
@@ -5097,6 +5455,7 @@
       <c r="F273" s="11" t="n"/>
       <c r="G273" s="11" t="n"/>
       <c r="H273" s="11" t="n"/>
+      <c r="I273" s="11" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="10">
@@ -5110,6 +5469,7 @@
       <c r="F274" s="11" t="n"/>
       <c r="G274" s="11" t="n"/>
       <c r="H274" s="11" t="n"/>
+      <c r="I274" s="11" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="10">
@@ -5123,6 +5483,7 @@
       <c r="F275" s="11" t="n"/>
       <c r="G275" s="11" t="n"/>
       <c r="H275" s="11" t="n"/>
+      <c r="I275" s="11" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="10">
@@ -5136,6 +5497,7 @@
       <c r="F276" s="11" t="n"/>
       <c r="G276" s="11" t="n"/>
       <c r="H276" s="11" t="n"/>
+      <c r="I276" s="11" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="10">
@@ -5149,6 +5511,7 @@
       <c r="F277" s="11" t="n"/>
       <c r="G277" s="11" t="n"/>
       <c r="H277" s="11" t="n"/>
+      <c r="I277" s="11" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="10">
@@ -5162,6 +5525,7 @@
       <c r="F278" s="11" t="n"/>
       <c r="G278" s="11" t="n"/>
       <c r="H278" s="11" t="n"/>
+      <c r="I278" s="11" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="10">
@@ -5175,6 +5539,7 @@
       <c r="F279" s="11" t="n"/>
       <c r="G279" s="11" t="n"/>
       <c r="H279" s="11" t="n"/>
+      <c r="I279" s="11" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="10">
@@ -5188,6 +5553,7 @@
       <c r="F280" s="11" t="n"/>
       <c r="G280" s="11" t="n"/>
       <c r="H280" s="11" t="n"/>
+      <c r="I280" s="11" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="10">
@@ -5201,6 +5567,7 @@
       <c r="F281" s="11" t="n"/>
       <c r="G281" s="11" t="n"/>
       <c r="H281" s="11" t="n"/>
+      <c r="I281" s="11" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="10">
@@ -5214,6 +5581,7 @@
       <c r="F282" s="11" t="n"/>
       <c r="G282" s="11" t="n"/>
       <c r="H282" s="11" t="n"/>
+      <c r="I282" s="11" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="10">
@@ -5227,6 +5595,7 @@
       <c r="F283" s="11" t="n"/>
       <c r="G283" s="11" t="n"/>
       <c r="H283" s="11" t="n"/>
+      <c r="I283" s="11" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="10">
@@ -5240,6 +5609,7 @@
       <c r="F284" s="11" t="n"/>
       <c r="G284" s="11" t="n"/>
       <c r="H284" s="11" t="n"/>
+      <c r="I284" s="11" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="10">
@@ -5253,6 +5623,7 @@
       <c r="F285" s="11" t="n"/>
       <c r="G285" s="11" t="n"/>
       <c r="H285" s="11" t="n"/>
+      <c r="I285" s="11" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="10">
@@ -5266,6 +5637,7 @@
       <c r="F286" s="11" t="n"/>
       <c r="G286" s="11" t="n"/>
       <c r="H286" s="11" t="n"/>
+      <c r="I286" s="11" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="10">
@@ -5279,6 +5651,7 @@
       <c r="F287" s="11" t="n"/>
       <c r="G287" s="11" t="n"/>
       <c r="H287" s="11" t="n"/>
+      <c r="I287" s="11" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="10">
@@ -5292,6 +5665,7 @@
       <c r="F288" s="11" t="n"/>
       <c r="G288" s="11" t="n"/>
       <c r="H288" s="11" t="n"/>
+      <c r="I288" s="11" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="10">
@@ -5305,6 +5679,7 @@
       <c r="F289" s="11" t="n"/>
       <c r="G289" s="11" t="n"/>
       <c r="H289" s="11" t="n"/>
+      <c r="I289" s="11" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="10">
@@ -5318,6 +5693,7 @@
       <c r="F290" s="11" t="n"/>
       <c r="G290" s="11" t="n"/>
       <c r="H290" s="11" t="n"/>
+      <c r="I290" s="11" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="10">
@@ -5331,6 +5707,7 @@
       <c r="F291" s="11" t="n"/>
       <c r="G291" s="11" t="n"/>
       <c r="H291" s="11" t="n"/>
+      <c r="I291" s="11" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="10">
@@ -5344,6 +5721,7 @@
       <c r="F292" s="11" t="n"/>
       <c r="G292" s="11" t="n"/>
       <c r="H292" s="11" t="n"/>
+      <c r="I292" s="11" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="10">
@@ -5357,6 +5735,7 @@
       <c r="F293" s="11" t="n"/>
       <c r="G293" s="11" t="n"/>
       <c r="H293" s="11" t="n"/>
+      <c r="I293" s="11" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="10">
@@ -5370,6 +5749,7 @@
       <c r="F294" s="11" t="n"/>
       <c r="G294" s="11" t="n"/>
       <c r="H294" s="11" t="n"/>
+      <c r="I294" s="11" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="10">
@@ -5383,6 +5763,7 @@
       <c r="F295" s="11" t="n"/>
       <c r="G295" s="11" t="n"/>
       <c r="H295" s="11" t="n"/>
+      <c r="I295" s="11" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="10">
@@ -5396,6 +5777,7 @@
       <c r="F296" s="11" t="n"/>
       <c r="G296" s="11" t="n"/>
       <c r="H296" s="11" t="n"/>
+      <c r="I296" s="11" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="10">
@@ -5409,6 +5791,7 @@
       <c r="F297" s="11" t="n"/>
       <c r="G297" s="11" t="n"/>
       <c r="H297" s="11" t="n"/>
+      <c r="I297" s="11" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="10">
@@ -5422,6 +5805,7 @@
       <c r="F298" s="11" t="n"/>
       <c r="G298" s="11" t="n"/>
       <c r="H298" s="11" t="n"/>
+      <c r="I298" s="11" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="10">
@@ -5435,6 +5819,7 @@
       <c r="F299" s="11" t="n"/>
       <c r="G299" s="11" t="n"/>
       <c r="H299" s="11" t="n"/>
+      <c r="I299" s="11" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="10">
@@ -5448,6 +5833,7 @@
       <c r="F300" s="11" t="n"/>
       <c r="G300" s="11" t="n"/>
       <c r="H300" s="11" t="n"/>
+      <c r="I300" s="11" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="10">
@@ -5461,6 +5847,7 @@
       <c r="F301" s="11" t="n"/>
       <c r="G301" s="11" t="n"/>
       <c r="H301" s="11" t="n"/>
+      <c r="I301" s="11" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="10">
@@ -5474,6 +5861,7 @@
       <c r="F302" s="11" t="n"/>
       <c r="G302" s="11" t="n"/>
       <c r="H302" s="11" t="n"/>
+      <c r="I302" s="11" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="10">
@@ -5487,6 +5875,7 @@
       <c r="F303" s="11" t="n"/>
       <c r="G303" s="11" t="n"/>
       <c r="H303" s="11" t="n"/>
+      <c r="I303" s="11" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="10">
@@ -5500,6 +5889,7 @@
       <c r="F304" s="11" t="n"/>
       <c r="G304" s="11" t="n"/>
       <c r="H304" s="11" t="n"/>
+      <c r="I304" s="11" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="10">
@@ -5513,6 +5903,7 @@
       <c r="F305" s="11" t="n"/>
       <c r="G305" s="11" t="n"/>
       <c r="H305" s="11" t="n"/>
+      <c r="I305" s="11" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="10">
@@ -5526,6 +5917,7 @@
       <c r="F306" s="11" t="n"/>
       <c r="G306" s="11" t="n"/>
       <c r="H306" s="11" t="n"/>
+      <c r="I306" s="11" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="10">
@@ -5539,6 +5931,7 @@
       <c r="F307" s="11" t="n"/>
       <c r="G307" s="11" t="n"/>
       <c r="H307" s="11" t="n"/>
+      <c r="I307" s="11" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="10">
@@ -5552,6 +5945,7 @@
       <c r="F308" s="11" t="n"/>
       <c r="G308" s="11" t="n"/>
       <c r="H308" s="11" t="n"/>
+      <c r="I308" s="11" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="10">
@@ -5565,6 +5959,7 @@
       <c r="F309" s="11" t="n"/>
       <c r="G309" s="11" t="n"/>
       <c r="H309" s="11" t="n"/>
+      <c r="I309" s="11" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="10">
@@ -5578,6 +5973,7 @@
       <c r="F310" s="11" t="n"/>
       <c r="G310" s="11" t="n"/>
       <c r="H310" s="11" t="n"/>
+      <c r="I310" s="11" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="10">
@@ -5591,9 +5987,15 @@
       <c r="F311" s="11" t="n"/>
       <c r="G311" s="11" t="n"/>
       <c r="H311" s="11" t="n"/>
+      <c r="I311" s="11" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:H311"/>
+  <autoFilter ref="A5:I311"/>
+  <dataValidations count="1">
+    <dataValidation sqref="I6:I311" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Achat-revente,Prestation de services"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Livre des recettes : ajoute la nature « Convoyage automobile » et son sous-total
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -1346,11 +1346,11 @@
       </c>
       <c r="K7" s="8" t="inlineStr">
         <is>
-          <t>URSSAF — 12,4 % revente · 21,3 % prestations (taux à confirmer)</t>
+          <t xml:space="preserve">  dont convoyage automobile</t>
         </is>
       </c>
       <c r="L7" s="9">
-        <f>L5*0.124+L6*0.213</f>
+        <f>SUMIF(I6:I311,"Convoyage automobile",E6:E311)</f>
         <v/>
       </c>
     </row>
@@ -1399,11 +1399,11 @@
       </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
-          <t>Reste après URSSAF</t>
+          <t>URSSAF — 12,4 % revente · 21,3 % prestations et convoyage (taux à confirmer)</t>
         </is>
       </c>
       <c r="L8" s="9">
-        <f>L4-L7</f>
+        <f>L5*0.124+(L6+L7)*0.213</f>
         <v/>
       </c>
     </row>
@@ -1449,6 +1449,15 @@
         <is>
           <t>Achat-revente</t>
         </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>Reste après URSSAF</t>
+        </is>
+      </c>
+      <c r="L9" s="9">
+        <f>L4-L8</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -5993,7 +6002,7 @@
   <autoFilter ref="A5:I311"/>
   <dataValidations count="1">
     <dataValidation sqref="I6:I311" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Achat-revente,Prestation de services"</formula1>
+      <formula1>"Achat-revente,Prestation de services,Convoyage automobile"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Livre des recettes : la prestation de 40 € correspond aux livraisons Uber (clients divers)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -1710,17 +1710,17 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>à compléter</t>
+          <t>3e trimestre 2026</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>à compléter</t>
+          <t>Divers clients</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Prestation de services commerciaux</t>
+          <t>Livraisons Uber — prestations de services diverses</t>
         </is>
       </c>
       <c r="E15" s="12" t="n">
@@ -1728,17 +1728,17 @@
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>à compléter</t>
+          <t>Virement Uber</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Déclarée au 3e trimestre 2026</t>
+          <t>Relevé de paiements Uber — déclaré au 3e trimestre 2026</t>
         </is>
       </c>
       <c r="I15" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Livre des recettes : premier encaissement de convoyage automobile (161,80 € le 22/10/2026)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -1757,14 +1757,44 @@
         <f>IF(B16="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="12" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
-      <c r="H16" s="11" t="n"/>
-      <c r="I16" s="11" t="n"/>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>à compléter</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Convoyage automobile — premières missions</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>161.8</v>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Virement</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>Relevé de missions — 4e trimestre 2026</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Convoyage automobile</t>
+        </is>
+      </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
           <t>Le CA déclaré est le montant ENCAISSÉ sur la période, pas facturé.</t>

</xml_diff>

<commit_message>
Livre des recettes : note sur le prélèvement direct de l'URSSAF par Uber à partir d'octobre 2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -1702,6 +1702,11 @@
           <t>Achat-revente</t>
         </is>
       </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>UBER : à partir du 4e trimestre 2026 (octobre), l'URSSAF est prélevée directement par Uber — ne pas la payer deux fois. Organisation à définir.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="10">

</xml_diff>

<commit_message>
Livre des recettes : le convoyage du 22/10 vient de la plateforme Hiflow
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -1769,7 +1769,7 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>à compléter</t>
+          <t>Hiflow</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1782,17 +1782,17 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Virement</t>
+          <t>Virement Hiflow</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Hiflow</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>Relevé de missions — 4e trimestre 2026</t>
+          <t>Relevé de missions Hiflow — 4e trimestre 2026</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Registres : colonne « Trimestre » et onglet « Par trimestre » (totaux par trimestre et par année)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -9,13 +9,14 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livre des recettes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registre des achats" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objets mobiliers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Par trimestre" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registre des achats" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objets mobiliers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Livre des recettes'!$A$5:$I$311</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Registre des achats'!$A$5:$G$350</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Objets mobiliers'!$A$5:$K$345</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Livre des recettes'!$A$5:$J$311</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Registre des achats'!$A$5:$G$350</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Objets mobiliers'!$A$5:$K$345</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +27,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00 &quot;€&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,8 +77,11 @@
       <color rgb="00C0392B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -92,6 +96,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF3EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
   </fills>
@@ -121,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -145,6 +154,9 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1150,7 +1162,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="32" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
     <col width="52" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
   </cols>
@@ -1238,6 +1250,11 @@
           <t>Nature de la recette</t>
         </is>
       </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Trimestre</t>
+        </is>
+      </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  dont achat-revente</t>
@@ -1291,6 +1308,10 @@
           <t>Achat-revente</t>
         </is>
       </c>
+      <c r="J6" s="11">
+        <f>IF(B6="","",IFERROR(RIGHT(B6,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B6,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  dont prestations de services</t>
@@ -1344,6 +1365,10 @@
           <t>Achat-revente</t>
         </is>
       </c>
+      <c r="J7" s="11">
+        <f>IF(B7="","",IFERROR(RIGHT(B7,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B7,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K7" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  dont convoyage automobile</t>
@@ -1397,6 +1422,10 @@
           <t>Achat-revente</t>
         </is>
       </c>
+      <c r="J8" s="11">
+        <f>IF(B8="","",IFERROR(RIGHT(B8,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B8,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
           <t>URSSAF — 12,4 % revente · 21,3 % prestations et convoyage (taux à confirmer)</t>
@@ -1450,6 +1479,10 @@
           <t>Achat-revente</t>
         </is>
       </c>
+      <c r="J9" s="11">
+        <f>IF(B9="","",IFERROR(RIGHT(B9,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B9,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K9" s="8" t="inlineStr">
         <is>
           <t>Reste après URSSAF</t>
@@ -1503,6 +1536,10 @@
           <t>Achat-revente</t>
         </is>
       </c>
+      <c r="J10" s="11">
+        <f>IF(B10="","",IFERROR(RIGHT(B10,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B10,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
           <t>EN ATTENTE D'ENCAISSEMENT</t>
@@ -1552,6 +1589,10 @@
           <t>Achat-revente</t>
         </is>
       </c>
+      <c r="J11" s="11">
+        <f>IF(B11="","",IFERROR(RIGHT(B11,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B11,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K11" s="8" t="inlineStr">
         <is>
           <t>BALLERINES MASSIMO DUTTI P.41 — vendues le 17/10/2026 sur Vinted à « anavdlr »</t>
@@ -1604,6 +1645,10 @@
           <t>Achat-revente</t>
         </is>
       </c>
+      <c r="J12" s="11">
+        <f>IF(B12="","",IFERROR(RIGHT(B12,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B12,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
           <t>Fonds retenus par Vinted. Relèvera du 4e trimestre 2026.</t>
@@ -1653,6 +1698,10 @@
           <t>Achat-revente</t>
         </is>
       </c>
+      <c r="J13" s="11">
+        <f>IF(B13="","",IFERROR(RIGHT(B13,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B13,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
           <t>À BASCULER dans le registre le jour du virement, pas avant.</t>
@@ -1702,6 +1751,10 @@
           <t>Achat-revente</t>
         </is>
       </c>
+      <c r="J14" s="11">
+        <f>IF(B14="","",IFERROR(RIGHT(B14,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B14,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
           <t>UBER : à partir du 4e trimestre 2026 (octobre), l'URSSAF est prélevée directement par Uber — ne pas la payer deux fois. Organisation à définir.</t>
@@ -1751,6 +1804,11 @@
           <t>Prestation de services</t>
         </is>
       </c>
+      <c r="J15" s="11" t="inlineStr">
+        <is>
+          <t>2026 T3</t>
+        </is>
+      </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
           <t>DÉCLARATION URSSAF</t>
@@ -1799,6 +1857,10 @@
         <is>
           <t>Convoyage automobile</t>
         </is>
+      </c>
+      <c r="J16" s="11">
+        <f>IF(B16="","",IFERROR(RIGHT(B16,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B16,4,2))/3,0),""))</f>
+        <v/>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
@@ -1819,6 +1881,10 @@
       <c r="G17" s="11" t="n"/>
       <c r="H17" s="11" t="n"/>
       <c r="I17" s="11" t="n"/>
+      <c r="J17" s="11">
+        <f>IF(B17="","",IFERROR(RIGHT(B17,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B17,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
           <t>Une vente d'août encaissée en septembre se déclare en septembre.</t>
@@ -1838,6 +1904,10 @@
       <c r="G18" s="11" t="n"/>
       <c r="H18" s="11" t="n"/>
       <c r="I18" s="11" t="n"/>
+      <c r="J18" s="11">
+        <f>IF(B18="","",IFERROR(RIGHT(B18,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B18,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
           <t>Filtrer la colonne « Date d'encaissement » pour isoler le trimestre.</t>
@@ -1857,6 +1927,10 @@
       <c r="G19" s="11" t="n"/>
       <c r="H19" s="11" t="n"/>
       <c r="I19" s="11" t="n"/>
+      <c r="J19" s="11">
+        <f>IF(B19="","",IFERROR(RIGHT(B19,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B19,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
           <t>3e trimestre 2026 : 627 € déclarés (587 € de revente + 40 € de prestation), 81 € d'URSSAF payés.</t>
@@ -1876,6 +1950,10 @@
       <c r="G20" s="11" t="n"/>
       <c r="H20" s="11" t="n"/>
       <c r="I20" s="11" t="n"/>
+      <c r="J20" s="11">
+        <f>IF(B20="","",IFERROR(RIGHT(B20,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B20,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
           <t>Les 206,82 € d'apports personnels n'en font PAS partie : ce ne sont pas des recettes.</t>
@@ -1895,6 +1973,10 @@
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="11" t="n"/>
       <c r="I21" s="11" t="n"/>
+      <c r="J21" s="11">
+        <f>IF(B21="","",IFERROR(RIGHT(B21,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B21,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
           <t>VENTES EN ESPÈCES — CE QU'IL FAUT GARDER</t>
@@ -1914,6 +1996,10 @@
       <c r="G22" s="11" t="n"/>
       <c r="H22" s="11" t="n"/>
       <c r="I22" s="11" t="n"/>
+      <c r="J22" s="11">
+        <f>IF(B22="","",IFERROR(RIGHT(B22,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B22,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
           <t>Légal sans limite entre un professionnel et un particulier résidant en France jusqu'à 1 000 €</t>
@@ -1933,6 +2019,10 @@
       <c r="G23" s="11" t="n"/>
       <c r="H23" s="11" t="n"/>
       <c r="I23" s="11" t="n"/>
+      <c r="J23" s="11">
+        <f>IF(B23="","",IFERROR(RIGHT(B23,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B23,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
           <t>par transaction (art. L112-6 du code monétaire et financier). Toutes les ventes sont loin du seuil.</t>
@@ -1952,6 +2042,10 @@
       <c r="G24" s="11" t="n"/>
       <c r="H24" s="11" t="n"/>
       <c r="I24" s="11" t="n"/>
+      <c r="J24" s="11">
+        <f>IF(B24="","",IFERROR(RIGHT(B24,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B24,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1967,6 +2061,10 @@
       <c r="G25" s="11" t="n"/>
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="11" t="n"/>
+      <c r="J25" s="11">
+        <f>IF(B25="","",IFERROR(RIGHT(B25,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B25,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
           <t>La preuve d'une vente en espèces, c'est le registre plus le dépôt bancaire. Trois réflexes :</t>
@@ -1986,6 +2084,10 @@
       <c r="G26" s="11" t="n"/>
       <c r="H26" s="11" t="n"/>
       <c r="I26" s="11" t="n"/>
+      <c r="J26" s="11">
+        <f>IF(B26="","",IFERROR(RIGHT(B26,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B26,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  1. Une note de vente par transaction — date, article, prix, nom de l'acheteur. Un carnet suffit.</t>
@@ -2005,6 +2107,10 @@
       <c r="G27" s="11" t="n"/>
       <c r="H27" s="11" t="n"/>
       <c r="I27" s="11" t="n"/>
+      <c r="J27" s="11">
+        <f>IF(B27="","",IFERROR(RIGHT(B27,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B27,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  2. Déposer sur le compte professionnel, pas sur le compte personnel : le détour brouille la piste.</t>
@@ -2024,6 +2130,10 @@
       <c r="G28" s="11" t="n"/>
       <c r="H28" s="11" t="n"/>
       <c r="I28" s="11" t="n"/>
+      <c r="J28" s="11">
+        <f>IF(B28="","",IFERROR(RIGHT(B28,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B28,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  3. Déposer par montants qui recoupent le registre, pour que le relevé confirme les lignes.</t>
@@ -2046,6 +2156,10 @@
       <c r="G29" s="11" t="n"/>
       <c r="H29" s="11" t="n"/>
       <c r="I29" s="11" t="n"/>
+      <c r="J29" s="11">
+        <f>IF(B29="","",IFERROR(RIGHT(B29,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B29,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K29" s="8" t="inlineStr">
         <is>
           <t>Baskets NIKE Air Max Moto 2K P.44.5 — gardées, 09/08/2026</t>
@@ -2068,6 +2182,10 @@
       <c r="G30" s="11" t="n"/>
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="11" t="n"/>
+      <c r="J30" s="11">
+        <f>IF(B30="","",IFERROR(RIGHT(B30,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B30,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K30" s="8" t="inlineStr">
         <is>
           <t>Pompe ROBBY VP550W ligne 131 — gardée, 26/07/2026</t>
@@ -2087,6 +2205,10 @@
       <c r="G31" s="11" t="n"/>
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="11" t="n"/>
+      <c r="J31" s="11">
+        <f>IF(B31="","",IFERROR(RIGHT(B31,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B31,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K31" s="8" t="inlineStr">
         <is>
           <t>Booster High Class MEGA Dream ex M2a — gardé, 03/08/2026</t>
@@ -2106,6 +2228,10 @@
       <c r="G32" s="11" t="n"/>
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="11" t="n"/>
+      <c r="J32" s="11">
+        <f>IF(B32="","",IFERROR(RIGHT(B32,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B32,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="10">
@@ -2120,6 +2246,10 @@
       <c r="G33" s="11" t="n"/>
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="11" t="n"/>
+      <c r="J33" s="11">
+        <f>IF(B33="","",IFERROR(RIGHT(B33,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B33,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
           <t>Un micro-entrepreneur ne peut pas se vendre à lui-même : il n'y a pas deux personnes juridiques.</t>
@@ -2139,6 +2269,10 @@
       <c r="G34" s="11" t="n"/>
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="11" t="n"/>
+      <c r="J34" s="11">
+        <f>IF(B34="","",IFERROR(RIGHT(B34,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B34,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
           <t>Reprendre un article pour soi n'est pas une recette — aucun chiffre d'affaires, donc aucune URSSAF.</t>
@@ -2158,6 +2292,10 @@
       <c r="G35" s="11" t="n"/>
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="11" t="n"/>
+      <c r="J35" s="11">
+        <f>IF(B35="","",IFERROR(RIGHT(B35,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B35,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
           <t>Verser de l'argent de son compte personnel vers le compte pro est un APPORT, pas un encaissement.</t>
@@ -2177,6 +2315,10 @@
       <c r="G36" s="11" t="n"/>
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="11" t="n"/>
+      <c r="J36" s="11">
+        <f>IF(B36="","",IFERROR(RIGHT(B36,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B36,4,2))/3,0),""))</f>
+        <v/>
+      </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
           <t>Ces lignes se notent en sortie au registre des objets mobiliers, jamais au livre des recettes.</t>
@@ -2196,6 +2338,10 @@
       <c r="G37" s="11" t="n"/>
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="11" t="n"/>
+      <c r="J37" s="11">
+        <f>IF(B37="","",IFERROR(RIGHT(B37,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B37,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="10">
@@ -2210,6 +2356,10 @@
       <c r="G38" s="11" t="n"/>
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="11" t="n"/>
+      <c r="J38" s="11">
+        <f>IF(B38="","",IFERROR(RIGHT(B38,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B38,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="10">
@@ -2224,6 +2374,10 @@
       <c r="G39" s="11" t="n"/>
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="11" t="n"/>
+      <c r="J39" s="11">
+        <f>IF(B39="","",IFERROR(RIGHT(B39,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B39,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="10">
@@ -2238,6 +2392,10 @@
       <c r="G40" s="11" t="n"/>
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="11" t="n"/>
+      <c r="J40" s="11">
+        <f>IF(B40="","",IFERROR(RIGHT(B40,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B40,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="10">
@@ -2252,6 +2410,10 @@
       <c r="G41" s="11" t="n"/>
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="11" t="n"/>
+      <c r="J41" s="11">
+        <f>IF(B41="","",IFERROR(RIGHT(B41,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B41,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="10">
@@ -2266,6 +2428,10 @@
       <c r="G42" s="11" t="n"/>
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="11" t="n"/>
+      <c r="J42" s="11">
+        <f>IF(B42="","",IFERROR(RIGHT(B42,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B42,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="10">
@@ -2280,6 +2446,10 @@
       <c r="G43" s="11" t="n"/>
       <c r="H43" s="11" t="n"/>
       <c r="I43" s="11" t="n"/>
+      <c r="J43" s="11">
+        <f>IF(B43="","",IFERROR(RIGHT(B43,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B43,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="10">
@@ -2294,6 +2464,10 @@
       <c r="G44" s="11" t="n"/>
       <c r="H44" s="11" t="n"/>
       <c r="I44" s="11" t="n"/>
+      <c r="J44" s="11">
+        <f>IF(B44="","",IFERROR(RIGHT(B44,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B44,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="10">
@@ -2308,6 +2482,10 @@
       <c r="G45" s="11" t="n"/>
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="11" t="n"/>
+      <c r="J45" s="11">
+        <f>IF(B45="","",IFERROR(RIGHT(B45,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B45,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="10">
@@ -2322,6 +2500,10 @@
       <c r="G46" s="11" t="n"/>
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="11" t="n"/>
+      <c r="J46" s="11">
+        <f>IF(B46="","",IFERROR(RIGHT(B46,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B46,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="10">
@@ -2336,6 +2518,10 @@
       <c r="G47" s="11" t="n"/>
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="11" t="n"/>
+      <c r="J47" s="11">
+        <f>IF(B47="","",IFERROR(RIGHT(B47,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B47,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="10">
@@ -2350,6 +2536,10 @@
       <c r="G48" s="11" t="n"/>
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="11" t="n"/>
+      <c r="J48" s="11">
+        <f>IF(B48="","",IFERROR(RIGHT(B48,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B48,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="10">
@@ -2364,6 +2554,10 @@
       <c r="G49" s="11" t="n"/>
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="11" t="n"/>
+      <c r="J49" s="11">
+        <f>IF(B49="","",IFERROR(RIGHT(B49,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B49,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="10">
@@ -2378,6 +2572,10 @@
       <c r="G50" s="11" t="n"/>
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="11" t="n"/>
+      <c r="J50" s="11">
+        <f>IF(B50="","",IFERROR(RIGHT(B50,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B50,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="10">
@@ -2392,6 +2590,10 @@
       <c r="G51" s="11" t="n"/>
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="11" t="n"/>
+      <c r="J51" s="11">
+        <f>IF(B51="","",IFERROR(RIGHT(B51,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B51,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="10">
@@ -2406,6 +2608,10 @@
       <c r="G52" s="11" t="n"/>
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="11" t="n"/>
+      <c r="J52" s="11">
+        <f>IF(B52="","",IFERROR(RIGHT(B52,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B52,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="10">
@@ -2420,6 +2626,10 @@
       <c r="G53" s="11" t="n"/>
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="11" t="n"/>
+      <c r="J53" s="11">
+        <f>IF(B53="","",IFERROR(RIGHT(B53,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B53,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="10">
@@ -2434,6 +2644,10 @@
       <c r="G54" s="11" t="n"/>
       <c r="H54" s="11" t="n"/>
       <c r="I54" s="11" t="n"/>
+      <c r="J54" s="11">
+        <f>IF(B54="","",IFERROR(RIGHT(B54,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B54,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="10">
@@ -2448,6 +2662,10 @@
       <c r="G55" s="11" t="n"/>
       <c r="H55" s="11" t="n"/>
       <c r="I55" s="11" t="n"/>
+      <c r="J55" s="11">
+        <f>IF(B55="","",IFERROR(RIGHT(B55,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B55,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="10">
@@ -2462,6 +2680,10 @@
       <c r="G56" s="11" t="n"/>
       <c r="H56" s="11" t="n"/>
       <c r="I56" s="11" t="n"/>
+      <c r="J56" s="11">
+        <f>IF(B56="","",IFERROR(RIGHT(B56,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B56,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="10">
@@ -2476,6 +2698,10 @@
       <c r="G57" s="11" t="n"/>
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="11" t="n"/>
+      <c r="J57" s="11">
+        <f>IF(B57="","",IFERROR(RIGHT(B57,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B57,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="10">
@@ -2490,6 +2716,10 @@
       <c r="G58" s="11" t="n"/>
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="11" t="n"/>
+      <c r="J58" s="11">
+        <f>IF(B58="","",IFERROR(RIGHT(B58,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B58,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="10">
@@ -2504,6 +2734,10 @@
       <c r="G59" s="11" t="n"/>
       <c r="H59" s="11" t="n"/>
       <c r="I59" s="11" t="n"/>
+      <c r="J59" s="11">
+        <f>IF(B59="","",IFERROR(RIGHT(B59,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B59,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="10">
@@ -2518,6 +2752,10 @@
       <c r="G60" s="11" t="n"/>
       <c r="H60" s="11" t="n"/>
       <c r="I60" s="11" t="n"/>
+      <c r="J60" s="11">
+        <f>IF(B60="","",IFERROR(RIGHT(B60,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B60,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="10">
@@ -2532,6 +2770,10 @@
       <c r="G61" s="11" t="n"/>
       <c r="H61" s="11" t="n"/>
       <c r="I61" s="11" t="n"/>
+      <c r="J61" s="11">
+        <f>IF(B61="","",IFERROR(RIGHT(B61,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B61,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="10">
@@ -2546,6 +2788,10 @@
       <c r="G62" s="11" t="n"/>
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="11" t="n"/>
+      <c r="J62" s="11">
+        <f>IF(B62="","",IFERROR(RIGHT(B62,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B62,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="10">
@@ -2560,6 +2806,10 @@
       <c r="G63" s="11" t="n"/>
       <c r="H63" s="11" t="n"/>
       <c r="I63" s="11" t="n"/>
+      <c r="J63" s="11">
+        <f>IF(B63="","",IFERROR(RIGHT(B63,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B63,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="10">
@@ -2574,6 +2824,10 @@
       <c r="G64" s="11" t="n"/>
       <c r="H64" s="11" t="n"/>
       <c r="I64" s="11" t="n"/>
+      <c r="J64" s="11">
+        <f>IF(B64="","",IFERROR(RIGHT(B64,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B64,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="10">
@@ -2588,6 +2842,10 @@
       <c r="G65" s="11" t="n"/>
       <c r="H65" s="11" t="n"/>
       <c r="I65" s="11" t="n"/>
+      <c r="J65" s="11">
+        <f>IF(B65="","",IFERROR(RIGHT(B65,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B65,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="10">
@@ -2602,6 +2860,10 @@
       <c r="G66" s="11" t="n"/>
       <c r="H66" s="11" t="n"/>
       <c r="I66" s="11" t="n"/>
+      <c r="J66" s="11">
+        <f>IF(B66="","",IFERROR(RIGHT(B66,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B66,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="10">
@@ -2616,6 +2878,10 @@
       <c r="G67" s="11" t="n"/>
       <c r="H67" s="11" t="n"/>
       <c r="I67" s="11" t="n"/>
+      <c r="J67" s="11">
+        <f>IF(B67="","",IFERROR(RIGHT(B67,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B67,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="10">
@@ -2630,6 +2896,10 @@
       <c r="G68" s="11" t="n"/>
       <c r="H68" s="11" t="n"/>
       <c r="I68" s="11" t="n"/>
+      <c r="J68" s="11">
+        <f>IF(B68="","",IFERROR(RIGHT(B68,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B68,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="10">
@@ -2644,6 +2914,10 @@
       <c r="G69" s="11" t="n"/>
       <c r="H69" s="11" t="n"/>
       <c r="I69" s="11" t="n"/>
+      <c r="J69" s="11">
+        <f>IF(B69="","",IFERROR(RIGHT(B69,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B69,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="10">
@@ -2658,6 +2932,10 @@
       <c r="G70" s="11" t="n"/>
       <c r="H70" s="11" t="n"/>
       <c r="I70" s="11" t="n"/>
+      <c r="J70" s="11">
+        <f>IF(B70="","",IFERROR(RIGHT(B70,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B70,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="10">
@@ -2672,6 +2950,10 @@
       <c r="G71" s="11" t="n"/>
       <c r="H71" s="11" t="n"/>
       <c r="I71" s="11" t="n"/>
+      <c r="J71" s="11">
+        <f>IF(B71="","",IFERROR(RIGHT(B71,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B71,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="10">
@@ -2686,6 +2968,10 @@
       <c r="G72" s="11" t="n"/>
       <c r="H72" s="11" t="n"/>
       <c r="I72" s="11" t="n"/>
+      <c r="J72" s="11">
+        <f>IF(B72="","",IFERROR(RIGHT(B72,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B72,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="10">
@@ -2700,6 +2986,10 @@
       <c r="G73" s="11" t="n"/>
       <c r="H73" s="11" t="n"/>
       <c r="I73" s="11" t="n"/>
+      <c r="J73" s="11">
+        <f>IF(B73="","",IFERROR(RIGHT(B73,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B73,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="10">
@@ -2714,6 +3004,10 @@
       <c r="G74" s="11" t="n"/>
       <c r="H74" s="11" t="n"/>
       <c r="I74" s="11" t="n"/>
+      <c r="J74" s="11">
+        <f>IF(B74="","",IFERROR(RIGHT(B74,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B74,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="10">
@@ -2728,6 +3022,10 @@
       <c r="G75" s="11" t="n"/>
       <c r="H75" s="11" t="n"/>
       <c r="I75" s="11" t="n"/>
+      <c r="J75" s="11">
+        <f>IF(B75="","",IFERROR(RIGHT(B75,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B75,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="10">
@@ -2742,6 +3040,10 @@
       <c r="G76" s="11" t="n"/>
       <c r="H76" s="11" t="n"/>
       <c r="I76" s="11" t="n"/>
+      <c r="J76" s="11">
+        <f>IF(B76="","",IFERROR(RIGHT(B76,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B76,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="10">
@@ -2756,6 +3058,10 @@
       <c r="G77" s="11" t="n"/>
       <c r="H77" s="11" t="n"/>
       <c r="I77" s="11" t="n"/>
+      <c r="J77" s="11">
+        <f>IF(B77="","",IFERROR(RIGHT(B77,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B77,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="10">
@@ -2770,6 +3076,10 @@
       <c r="G78" s="11" t="n"/>
       <c r="H78" s="11" t="n"/>
       <c r="I78" s="11" t="n"/>
+      <c r="J78" s="11">
+        <f>IF(B78="","",IFERROR(RIGHT(B78,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B78,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="10">
@@ -2784,6 +3094,10 @@
       <c r="G79" s="11" t="n"/>
       <c r="H79" s="11" t="n"/>
       <c r="I79" s="11" t="n"/>
+      <c r="J79" s="11">
+        <f>IF(B79="","",IFERROR(RIGHT(B79,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B79,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="10">
@@ -2798,6 +3112,10 @@
       <c r="G80" s="11" t="n"/>
       <c r="H80" s="11" t="n"/>
       <c r="I80" s="11" t="n"/>
+      <c r="J80" s="11">
+        <f>IF(B80="","",IFERROR(RIGHT(B80,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B80,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="10">
@@ -2812,6 +3130,10 @@
       <c r="G81" s="11" t="n"/>
       <c r="H81" s="11" t="n"/>
       <c r="I81" s="11" t="n"/>
+      <c r="J81" s="11">
+        <f>IF(B81="","",IFERROR(RIGHT(B81,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B81,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="10">
@@ -2826,6 +3148,10 @@
       <c r="G82" s="11" t="n"/>
       <c r="H82" s="11" t="n"/>
       <c r="I82" s="11" t="n"/>
+      <c r="J82" s="11">
+        <f>IF(B82="","",IFERROR(RIGHT(B82,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B82,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="10">
@@ -2840,6 +3166,10 @@
       <c r="G83" s="11" t="n"/>
       <c r="H83" s="11" t="n"/>
       <c r="I83" s="11" t="n"/>
+      <c r="J83" s="11">
+        <f>IF(B83="","",IFERROR(RIGHT(B83,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B83,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="10">
@@ -2854,6 +3184,10 @@
       <c r="G84" s="11" t="n"/>
       <c r="H84" s="11" t="n"/>
       <c r="I84" s="11" t="n"/>
+      <c r="J84" s="11">
+        <f>IF(B84="","",IFERROR(RIGHT(B84,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B84,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="10">
@@ -2868,6 +3202,10 @@
       <c r="G85" s="11" t="n"/>
       <c r="H85" s="11" t="n"/>
       <c r="I85" s="11" t="n"/>
+      <c r="J85" s="11">
+        <f>IF(B85="","",IFERROR(RIGHT(B85,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B85,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="10">
@@ -2882,6 +3220,10 @@
       <c r="G86" s="11" t="n"/>
       <c r="H86" s="11" t="n"/>
       <c r="I86" s="11" t="n"/>
+      <c r="J86" s="11">
+        <f>IF(B86="","",IFERROR(RIGHT(B86,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B86,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="10">
@@ -2896,6 +3238,10 @@
       <c r="G87" s="11" t="n"/>
       <c r="H87" s="11" t="n"/>
       <c r="I87" s="11" t="n"/>
+      <c r="J87" s="11">
+        <f>IF(B87="","",IFERROR(RIGHT(B87,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B87,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="10">
@@ -2910,6 +3256,10 @@
       <c r="G88" s="11" t="n"/>
       <c r="H88" s="11" t="n"/>
       <c r="I88" s="11" t="n"/>
+      <c r="J88" s="11">
+        <f>IF(B88="","",IFERROR(RIGHT(B88,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B88,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="10">
@@ -2924,6 +3274,10 @@
       <c r="G89" s="11" t="n"/>
       <c r="H89" s="11" t="n"/>
       <c r="I89" s="11" t="n"/>
+      <c r="J89" s="11">
+        <f>IF(B89="","",IFERROR(RIGHT(B89,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B89,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="10">
@@ -2938,6 +3292,10 @@
       <c r="G90" s="11" t="n"/>
       <c r="H90" s="11" t="n"/>
       <c r="I90" s="11" t="n"/>
+      <c r="J90" s="11">
+        <f>IF(B90="","",IFERROR(RIGHT(B90,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B90,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="10">
@@ -2952,6 +3310,10 @@
       <c r="G91" s="11" t="n"/>
       <c r="H91" s="11" t="n"/>
       <c r="I91" s="11" t="n"/>
+      <c r="J91" s="11">
+        <f>IF(B91="","",IFERROR(RIGHT(B91,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B91,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="10">
@@ -2966,6 +3328,10 @@
       <c r="G92" s="11" t="n"/>
       <c r="H92" s="11" t="n"/>
       <c r="I92" s="11" t="n"/>
+      <c r="J92" s="11">
+        <f>IF(B92="","",IFERROR(RIGHT(B92,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B92,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="10">
@@ -2980,6 +3346,10 @@
       <c r="G93" s="11" t="n"/>
       <c r="H93" s="11" t="n"/>
       <c r="I93" s="11" t="n"/>
+      <c r="J93" s="11">
+        <f>IF(B93="","",IFERROR(RIGHT(B93,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B93,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="10">
@@ -2994,6 +3364,10 @@
       <c r="G94" s="11" t="n"/>
       <c r="H94" s="11" t="n"/>
       <c r="I94" s="11" t="n"/>
+      <c r="J94" s="11">
+        <f>IF(B94="","",IFERROR(RIGHT(B94,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B94,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="10">
@@ -3008,6 +3382,10 @@
       <c r="G95" s="11" t="n"/>
       <c r="H95" s="11" t="n"/>
       <c r="I95" s="11" t="n"/>
+      <c r="J95" s="11">
+        <f>IF(B95="","",IFERROR(RIGHT(B95,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B95,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="10">
@@ -3022,6 +3400,10 @@
       <c r="G96" s="11" t="n"/>
       <c r="H96" s="11" t="n"/>
       <c r="I96" s="11" t="n"/>
+      <c r="J96" s="11">
+        <f>IF(B96="","",IFERROR(RIGHT(B96,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B96,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="10">
@@ -3036,6 +3418,10 @@
       <c r="G97" s="11" t="n"/>
       <c r="H97" s="11" t="n"/>
       <c r="I97" s="11" t="n"/>
+      <c r="J97" s="11">
+        <f>IF(B97="","",IFERROR(RIGHT(B97,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B97,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="10">
@@ -3050,6 +3436,10 @@
       <c r="G98" s="11" t="n"/>
       <c r="H98" s="11" t="n"/>
       <c r="I98" s="11" t="n"/>
+      <c r="J98" s="11">
+        <f>IF(B98="","",IFERROR(RIGHT(B98,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B98,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="10">
@@ -3064,6 +3454,10 @@
       <c r="G99" s="11" t="n"/>
       <c r="H99" s="11" t="n"/>
       <c r="I99" s="11" t="n"/>
+      <c r="J99" s="11">
+        <f>IF(B99="","",IFERROR(RIGHT(B99,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B99,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="10">
@@ -3078,6 +3472,10 @@
       <c r="G100" s="11" t="n"/>
       <c r="H100" s="11" t="n"/>
       <c r="I100" s="11" t="n"/>
+      <c r="J100" s="11">
+        <f>IF(B100="","",IFERROR(RIGHT(B100,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B100,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="10">
@@ -3092,6 +3490,10 @@
       <c r="G101" s="11" t="n"/>
       <c r="H101" s="11" t="n"/>
       <c r="I101" s="11" t="n"/>
+      <c r="J101" s="11">
+        <f>IF(B101="","",IFERROR(RIGHT(B101,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B101,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="10">
@@ -3106,6 +3508,10 @@
       <c r="G102" s="11" t="n"/>
       <c r="H102" s="11" t="n"/>
       <c r="I102" s="11" t="n"/>
+      <c r="J102" s="11">
+        <f>IF(B102="","",IFERROR(RIGHT(B102,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B102,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="10">
@@ -3120,6 +3526,10 @@
       <c r="G103" s="11" t="n"/>
       <c r="H103" s="11" t="n"/>
       <c r="I103" s="11" t="n"/>
+      <c r="J103" s="11">
+        <f>IF(B103="","",IFERROR(RIGHT(B103,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B103,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="10">
@@ -3134,6 +3544,10 @@
       <c r="G104" s="11" t="n"/>
       <c r="H104" s="11" t="n"/>
       <c r="I104" s="11" t="n"/>
+      <c r="J104" s="11">
+        <f>IF(B104="","",IFERROR(RIGHT(B104,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B104,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="10">
@@ -3148,6 +3562,10 @@
       <c r="G105" s="11" t="n"/>
       <c r="H105" s="11" t="n"/>
       <c r="I105" s="11" t="n"/>
+      <c r="J105" s="11">
+        <f>IF(B105="","",IFERROR(RIGHT(B105,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B105,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="10">
@@ -3162,6 +3580,10 @@
       <c r="G106" s="11" t="n"/>
       <c r="H106" s="11" t="n"/>
       <c r="I106" s="11" t="n"/>
+      <c r="J106" s="11">
+        <f>IF(B106="","",IFERROR(RIGHT(B106,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B106,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="10">
@@ -3176,6 +3598,10 @@
       <c r="G107" s="11" t="n"/>
       <c r="H107" s="11" t="n"/>
       <c r="I107" s="11" t="n"/>
+      <c r="J107" s="11">
+        <f>IF(B107="","",IFERROR(RIGHT(B107,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B107,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="10">
@@ -3190,6 +3616,10 @@
       <c r="G108" s="11" t="n"/>
       <c r="H108" s="11" t="n"/>
       <c r="I108" s="11" t="n"/>
+      <c r="J108" s="11">
+        <f>IF(B108="","",IFERROR(RIGHT(B108,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B108,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="10">
@@ -3204,6 +3634,10 @@
       <c r="G109" s="11" t="n"/>
       <c r="H109" s="11" t="n"/>
       <c r="I109" s="11" t="n"/>
+      <c r="J109" s="11">
+        <f>IF(B109="","",IFERROR(RIGHT(B109,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B109,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="10">
@@ -3218,6 +3652,10 @@
       <c r="G110" s="11" t="n"/>
       <c r="H110" s="11" t="n"/>
       <c r="I110" s="11" t="n"/>
+      <c r="J110" s="11">
+        <f>IF(B110="","",IFERROR(RIGHT(B110,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B110,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="10">
@@ -3232,6 +3670,10 @@
       <c r="G111" s="11" t="n"/>
       <c r="H111" s="11" t="n"/>
       <c r="I111" s="11" t="n"/>
+      <c r="J111" s="11">
+        <f>IF(B111="","",IFERROR(RIGHT(B111,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B111,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="10">
@@ -3246,6 +3688,10 @@
       <c r="G112" s="11" t="n"/>
       <c r="H112" s="11" t="n"/>
       <c r="I112" s="11" t="n"/>
+      <c r="J112" s="11">
+        <f>IF(B112="","",IFERROR(RIGHT(B112,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B112,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="10">
@@ -3260,6 +3706,10 @@
       <c r="G113" s="11" t="n"/>
       <c r="H113" s="11" t="n"/>
       <c r="I113" s="11" t="n"/>
+      <c r="J113" s="11">
+        <f>IF(B113="","",IFERROR(RIGHT(B113,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B113,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="10">
@@ -3274,6 +3724,10 @@
       <c r="G114" s="11" t="n"/>
       <c r="H114" s="11" t="n"/>
       <c r="I114" s="11" t="n"/>
+      <c r="J114" s="11">
+        <f>IF(B114="","",IFERROR(RIGHT(B114,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B114,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="10">
@@ -3288,6 +3742,10 @@
       <c r="G115" s="11" t="n"/>
       <c r="H115" s="11" t="n"/>
       <c r="I115" s="11" t="n"/>
+      <c r="J115" s="11">
+        <f>IF(B115="","",IFERROR(RIGHT(B115,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B115,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="10">
@@ -3302,6 +3760,10 @@
       <c r="G116" s="11" t="n"/>
       <c r="H116" s="11" t="n"/>
       <c r="I116" s="11" t="n"/>
+      <c r="J116" s="11">
+        <f>IF(B116="","",IFERROR(RIGHT(B116,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B116,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="10">
@@ -3316,6 +3778,10 @@
       <c r="G117" s="11" t="n"/>
       <c r="H117" s="11" t="n"/>
       <c r="I117" s="11" t="n"/>
+      <c r="J117" s="11">
+        <f>IF(B117="","",IFERROR(RIGHT(B117,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B117,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="10">
@@ -3330,6 +3796,10 @@
       <c r="G118" s="11" t="n"/>
       <c r="H118" s="11" t="n"/>
       <c r="I118" s="11" t="n"/>
+      <c r="J118" s="11">
+        <f>IF(B118="","",IFERROR(RIGHT(B118,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B118,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="10">
@@ -3344,6 +3814,10 @@
       <c r="G119" s="11" t="n"/>
       <c r="H119" s="11" t="n"/>
       <c r="I119" s="11" t="n"/>
+      <c r="J119" s="11">
+        <f>IF(B119="","",IFERROR(RIGHT(B119,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B119,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="10">
@@ -3358,6 +3832,10 @@
       <c r="G120" s="11" t="n"/>
       <c r="H120" s="11" t="n"/>
       <c r="I120" s="11" t="n"/>
+      <c r="J120" s="11">
+        <f>IF(B120="","",IFERROR(RIGHT(B120,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B120,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="10">
@@ -3372,6 +3850,10 @@
       <c r="G121" s="11" t="n"/>
       <c r="H121" s="11" t="n"/>
       <c r="I121" s="11" t="n"/>
+      <c r="J121" s="11">
+        <f>IF(B121="","",IFERROR(RIGHT(B121,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B121,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="10">
@@ -3386,6 +3868,10 @@
       <c r="G122" s="11" t="n"/>
       <c r="H122" s="11" t="n"/>
       <c r="I122" s="11" t="n"/>
+      <c r="J122" s="11">
+        <f>IF(B122="","",IFERROR(RIGHT(B122,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B122,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="10">
@@ -3400,6 +3886,10 @@
       <c r="G123" s="11" t="n"/>
       <c r="H123" s="11" t="n"/>
       <c r="I123" s="11" t="n"/>
+      <c r="J123" s="11">
+        <f>IF(B123="","",IFERROR(RIGHT(B123,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B123,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="10">
@@ -3414,6 +3904,10 @@
       <c r="G124" s="11" t="n"/>
       <c r="H124" s="11" t="n"/>
       <c r="I124" s="11" t="n"/>
+      <c r="J124" s="11">
+        <f>IF(B124="","",IFERROR(RIGHT(B124,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B124,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="10">
@@ -3428,6 +3922,10 @@
       <c r="G125" s="11" t="n"/>
       <c r="H125" s="11" t="n"/>
       <c r="I125" s="11" t="n"/>
+      <c r="J125" s="11">
+        <f>IF(B125="","",IFERROR(RIGHT(B125,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B125,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="10">
@@ -3442,6 +3940,10 @@
       <c r="G126" s="11" t="n"/>
       <c r="H126" s="11" t="n"/>
       <c r="I126" s="11" t="n"/>
+      <c r="J126" s="11">
+        <f>IF(B126="","",IFERROR(RIGHT(B126,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B126,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="10">
@@ -3456,6 +3958,10 @@
       <c r="G127" s="11" t="n"/>
       <c r="H127" s="11" t="n"/>
       <c r="I127" s="11" t="n"/>
+      <c r="J127" s="11">
+        <f>IF(B127="","",IFERROR(RIGHT(B127,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B127,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="10">
@@ -3470,6 +3976,10 @@
       <c r="G128" s="11" t="n"/>
       <c r="H128" s="11" t="n"/>
       <c r="I128" s="11" t="n"/>
+      <c r="J128" s="11">
+        <f>IF(B128="","",IFERROR(RIGHT(B128,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B128,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="10">
@@ -3484,6 +3994,10 @@
       <c r="G129" s="11" t="n"/>
       <c r="H129" s="11" t="n"/>
       <c r="I129" s="11" t="n"/>
+      <c r="J129" s="11">
+        <f>IF(B129="","",IFERROR(RIGHT(B129,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B129,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="10">
@@ -3498,6 +4012,10 @@
       <c r="G130" s="11" t="n"/>
       <c r="H130" s="11" t="n"/>
       <c r="I130" s="11" t="n"/>
+      <c r="J130" s="11">
+        <f>IF(B130="","",IFERROR(RIGHT(B130,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B130,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="10">
@@ -3512,6 +4030,10 @@
       <c r="G131" s="11" t="n"/>
       <c r="H131" s="11" t="n"/>
       <c r="I131" s="11" t="n"/>
+      <c r="J131" s="11">
+        <f>IF(B131="","",IFERROR(RIGHT(B131,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B131,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="10">
@@ -3526,6 +4048,10 @@
       <c r="G132" s="11" t="n"/>
       <c r="H132" s="11" t="n"/>
       <c r="I132" s="11" t="n"/>
+      <c r="J132" s="11">
+        <f>IF(B132="","",IFERROR(RIGHT(B132,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B132,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="10">
@@ -3540,6 +4066,10 @@
       <c r="G133" s="11" t="n"/>
       <c r="H133" s="11" t="n"/>
       <c r="I133" s="11" t="n"/>
+      <c r="J133" s="11">
+        <f>IF(B133="","",IFERROR(RIGHT(B133,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B133,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="10">
@@ -3554,6 +4084,10 @@
       <c r="G134" s="11" t="n"/>
       <c r="H134" s="11" t="n"/>
       <c r="I134" s="11" t="n"/>
+      <c r="J134" s="11">
+        <f>IF(B134="","",IFERROR(RIGHT(B134,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B134,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="10">
@@ -3568,6 +4102,10 @@
       <c r="G135" s="11" t="n"/>
       <c r="H135" s="11" t="n"/>
       <c r="I135" s="11" t="n"/>
+      <c r="J135" s="11">
+        <f>IF(B135="","",IFERROR(RIGHT(B135,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B135,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="10">
@@ -3582,6 +4120,10 @@
       <c r="G136" s="11" t="n"/>
       <c r="H136" s="11" t="n"/>
       <c r="I136" s="11" t="n"/>
+      <c r="J136" s="11">
+        <f>IF(B136="","",IFERROR(RIGHT(B136,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B136,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="10">
@@ -3596,6 +4138,10 @@
       <c r="G137" s="11" t="n"/>
       <c r="H137" s="11" t="n"/>
       <c r="I137" s="11" t="n"/>
+      <c r="J137" s="11">
+        <f>IF(B137="","",IFERROR(RIGHT(B137,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B137,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="10">
@@ -3610,6 +4156,10 @@
       <c r="G138" s="11" t="n"/>
       <c r="H138" s="11" t="n"/>
       <c r="I138" s="11" t="n"/>
+      <c r="J138" s="11">
+        <f>IF(B138="","",IFERROR(RIGHT(B138,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B138,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="10">
@@ -3624,6 +4174,10 @@
       <c r="G139" s="11" t="n"/>
       <c r="H139" s="11" t="n"/>
       <c r="I139" s="11" t="n"/>
+      <c r="J139" s="11">
+        <f>IF(B139="","",IFERROR(RIGHT(B139,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B139,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="10">
@@ -3638,6 +4192,10 @@
       <c r="G140" s="11" t="n"/>
       <c r="H140" s="11" t="n"/>
       <c r="I140" s="11" t="n"/>
+      <c r="J140" s="11">
+        <f>IF(B140="","",IFERROR(RIGHT(B140,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B140,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="10">
@@ -3652,6 +4210,10 @@
       <c r="G141" s="11" t="n"/>
       <c r="H141" s="11" t="n"/>
       <c r="I141" s="11" t="n"/>
+      <c r="J141" s="11">
+        <f>IF(B141="","",IFERROR(RIGHT(B141,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B141,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="10">
@@ -3666,6 +4228,10 @@
       <c r="G142" s="11" t="n"/>
       <c r="H142" s="11" t="n"/>
       <c r="I142" s="11" t="n"/>
+      <c r="J142" s="11">
+        <f>IF(B142="","",IFERROR(RIGHT(B142,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B142,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="10">
@@ -3680,6 +4246,10 @@
       <c r="G143" s="11" t="n"/>
       <c r="H143" s="11" t="n"/>
       <c r="I143" s="11" t="n"/>
+      <c r="J143" s="11">
+        <f>IF(B143="","",IFERROR(RIGHT(B143,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B143,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="10">
@@ -3694,6 +4264,10 @@
       <c r="G144" s="11" t="n"/>
       <c r="H144" s="11" t="n"/>
       <c r="I144" s="11" t="n"/>
+      <c r="J144" s="11">
+        <f>IF(B144="","",IFERROR(RIGHT(B144,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B144,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="10">
@@ -3708,6 +4282,10 @@
       <c r="G145" s="11" t="n"/>
       <c r="H145" s="11" t="n"/>
       <c r="I145" s="11" t="n"/>
+      <c r="J145" s="11">
+        <f>IF(B145="","",IFERROR(RIGHT(B145,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B145,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="10">
@@ -3722,6 +4300,10 @@
       <c r="G146" s="11" t="n"/>
       <c r="H146" s="11" t="n"/>
       <c r="I146" s="11" t="n"/>
+      <c r="J146" s="11">
+        <f>IF(B146="","",IFERROR(RIGHT(B146,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B146,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="10">
@@ -3736,6 +4318,10 @@
       <c r="G147" s="11" t="n"/>
       <c r="H147" s="11" t="n"/>
       <c r="I147" s="11" t="n"/>
+      <c r="J147" s="11">
+        <f>IF(B147="","",IFERROR(RIGHT(B147,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B147,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="10">
@@ -3750,6 +4336,10 @@
       <c r="G148" s="11" t="n"/>
       <c r="H148" s="11" t="n"/>
       <c r="I148" s="11" t="n"/>
+      <c r="J148" s="11">
+        <f>IF(B148="","",IFERROR(RIGHT(B148,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B148,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="10">
@@ -3764,6 +4354,10 @@
       <c r="G149" s="11" t="n"/>
       <c r="H149" s="11" t="n"/>
       <c r="I149" s="11" t="n"/>
+      <c r="J149" s="11">
+        <f>IF(B149="","",IFERROR(RIGHT(B149,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B149,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="10">
@@ -3778,6 +4372,10 @@
       <c r="G150" s="11" t="n"/>
       <c r="H150" s="11" t="n"/>
       <c r="I150" s="11" t="n"/>
+      <c r="J150" s="11">
+        <f>IF(B150="","",IFERROR(RIGHT(B150,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B150,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="10">
@@ -3792,6 +4390,10 @@
       <c r="G151" s="11" t="n"/>
       <c r="H151" s="11" t="n"/>
       <c r="I151" s="11" t="n"/>
+      <c r="J151" s="11">
+        <f>IF(B151="","",IFERROR(RIGHT(B151,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B151,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="10">
@@ -3806,6 +4408,10 @@
       <c r="G152" s="11" t="n"/>
       <c r="H152" s="11" t="n"/>
       <c r="I152" s="11" t="n"/>
+      <c r="J152" s="11">
+        <f>IF(B152="","",IFERROR(RIGHT(B152,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B152,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="10">
@@ -3820,6 +4426,10 @@
       <c r="G153" s="11" t="n"/>
       <c r="H153" s="11" t="n"/>
       <c r="I153" s="11" t="n"/>
+      <c r="J153" s="11">
+        <f>IF(B153="","",IFERROR(RIGHT(B153,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B153,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="10">
@@ -3834,6 +4444,10 @@
       <c r="G154" s="11" t="n"/>
       <c r="H154" s="11" t="n"/>
       <c r="I154" s="11" t="n"/>
+      <c r="J154" s="11">
+        <f>IF(B154="","",IFERROR(RIGHT(B154,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B154,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="10">
@@ -3848,6 +4462,10 @@
       <c r="G155" s="11" t="n"/>
       <c r="H155" s="11" t="n"/>
       <c r="I155" s="11" t="n"/>
+      <c r="J155" s="11">
+        <f>IF(B155="","",IFERROR(RIGHT(B155,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B155,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="10">
@@ -3862,6 +4480,10 @@
       <c r="G156" s="11" t="n"/>
       <c r="H156" s="11" t="n"/>
       <c r="I156" s="11" t="n"/>
+      <c r="J156" s="11">
+        <f>IF(B156="","",IFERROR(RIGHT(B156,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B156,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="10">
@@ -3876,6 +4498,10 @@
       <c r="G157" s="11" t="n"/>
       <c r="H157" s="11" t="n"/>
       <c r="I157" s="11" t="n"/>
+      <c r="J157" s="11">
+        <f>IF(B157="","",IFERROR(RIGHT(B157,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B157,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="10">
@@ -3890,6 +4516,10 @@
       <c r="G158" s="11" t="n"/>
       <c r="H158" s="11" t="n"/>
       <c r="I158" s="11" t="n"/>
+      <c r="J158" s="11">
+        <f>IF(B158="","",IFERROR(RIGHT(B158,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B158,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="10">
@@ -3904,6 +4534,10 @@
       <c r="G159" s="11" t="n"/>
       <c r="H159" s="11" t="n"/>
       <c r="I159" s="11" t="n"/>
+      <c r="J159" s="11">
+        <f>IF(B159="","",IFERROR(RIGHT(B159,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B159,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="10">
@@ -3918,6 +4552,10 @@
       <c r="G160" s="11" t="n"/>
       <c r="H160" s="11" t="n"/>
       <c r="I160" s="11" t="n"/>
+      <c r="J160" s="11">
+        <f>IF(B160="","",IFERROR(RIGHT(B160,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B160,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="10">
@@ -3932,6 +4570,10 @@
       <c r="G161" s="11" t="n"/>
       <c r="H161" s="11" t="n"/>
       <c r="I161" s="11" t="n"/>
+      <c r="J161" s="11">
+        <f>IF(B161="","",IFERROR(RIGHT(B161,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B161,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="10">
@@ -3946,6 +4588,10 @@
       <c r="G162" s="11" t="n"/>
       <c r="H162" s="11" t="n"/>
       <c r="I162" s="11" t="n"/>
+      <c r="J162" s="11">
+        <f>IF(B162="","",IFERROR(RIGHT(B162,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B162,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="10">
@@ -3960,6 +4606,10 @@
       <c r="G163" s="11" t="n"/>
       <c r="H163" s="11" t="n"/>
       <c r="I163" s="11" t="n"/>
+      <c r="J163" s="11">
+        <f>IF(B163="","",IFERROR(RIGHT(B163,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B163,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="10">
@@ -3974,6 +4624,10 @@
       <c r="G164" s="11" t="n"/>
       <c r="H164" s="11" t="n"/>
       <c r="I164" s="11" t="n"/>
+      <c r="J164" s="11">
+        <f>IF(B164="","",IFERROR(RIGHT(B164,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B164,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="10">
@@ -3988,6 +4642,10 @@
       <c r="G165" s="11" t="n"/>
       <c r="H165" s="11" t="n"/>
       <c r="I165" s="11" t="n"/>
+      <c r="J165" s="11">
+        <f>IF(B165="","",IFERROR(RIGHT(B165,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B165,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="10">
@@ -4002,6 +4660,10 @@
       <c r="G166" s="11" t="n"/>
       <c r="H166" s="11" t="n"/>
       <c r="I166" s="11" t="n"/>
+      <c r="J166" s="11">
+        <f>IF(B166="","",IFERROR(RIGHT(B166,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B166,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="10">
@@ -4016,6 +4678,10 @@
       <c r="G167" s="11" t="n"/>
       <c r="H167" s="11" t="n"/>
       <c r="I167" s="11" t="n"/>
+      <c r="J167" s="11">
+        <f>IF(B167="","",IFERROR(RIGHT(B167,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B167,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="10">
@@ -4030,6 +4696,10 @@
       <c r="G168" s="11" t="n"/>
       <c r="H168" s="11" t="n"/>
       <c r="I168" s="11" t="n"/>
+      <c r="J168" s="11">
+        <f>IF(B168="","",IFERROR(RIGHT(B168,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B168,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="10">
@@ -4044,6 +4714,10 @@
       <c r="G169" s="11" t="n"/>
       <c r="H169" s="11" t="n"/>
       <c r="I169" s="11" t="n"/>
+      <c r="J169" s="11">
+        <f>IF(B169="","",IFERROR(RIGHT(B169,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B169,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="10">
@@ -4058,6 +4732,10 @@
       <c r="G170" s="11" t="n"/>
       <c r="H170" s="11" t="n"/>
       <c r="I170" s="11" t="n"/>
+      <c r="J170" s="11">
+        <f>IF(B170="","",IFERROR(RIGHT(B170,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B170,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="10">
@@ -4072,6 +4750,10 @@
       <c r="G171" s="11" t="n"/>
       <c r="H171" s="11" t="n"/>
       <c r="I171" s="11" t="n"/>
+      <c r="J171" s="11">
+        <f>IF(B171="","",IFERROR(RIGHT(B171,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B171,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="10">
@@ -4086,6 +4768,10 @@
       <c r="G172" s="11" t="n"/>
       <c r="H172" s="11" t="n"/>
       <c r="I172" s="11" t="n"/>
+      <c r="J172" s="11">
+        <f>IF(B172="","",IFERROR(RIGHT(B172,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B172,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="10">
@@ -4100,6 +4786,10 @@
       <c r="G173" s="11" t="n"/>
       <c r="H173" s="11" t="n"/>
       <c r="I173" s="11" t="n"/>
+      <c r="J173" s="11">
+        <f>IF(B173="","",IFERROR(RIGHT(B173,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B173,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="10">
@@ -4114,6 +4804,10 @@
       <c r="G174" s="11" t="n"/>
       <c r="H174" s="11" t="n"/>
       <c r="I174" s="11" t="n"/>
+      <c r="J174" s="11">
+        <f>IF(B174="","",IFERROR(RIGHT(B174,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B174,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="10">
@@ -4128,6 +4822,10 @@
       <c r="G175" s="11" t="n"/>
       <c r="H175" s="11" t="n"/>
       <c r="I175" s="11" t="n"/>
+      <c r="J175" s="11">
+        <f>IF(B175="","",IFERROR(RIGHT(B175,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B175,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="10">
@@ -4142,6 +4840,10 @@
       <c r="G176" s="11" t="n"/>
       <c r="H176" s="11" t="n"/>
       <c r="I176" s="11" t="n"/>
+      <c r="J176" s="11">
+        <f>IF(B176="","",IFERROR(RIGHT(B176,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B176,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="10">
@@ -4156,6 +4858,10 @@
       <c r="G177" s="11" t="n"/>
       <c r="H177" s="11" t="n"/>
       <c r="I177" s="11" t="n"/>
+      <c r="J177" s="11">
+        <f>IF(B177="","",IFERROR(RIGHT(B177,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B177,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="10">
@@ -4170,6 +4876,10 @@
       <c r="G178" s="11" t="n"/>
       <c r="H178" s="11" t="n"/>
       <c r="I178" s="11" t="n"/>
+      <c r="J178" s="11">
+        <f>IF(B178="","",IFERROR(RIGHT(B178,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B178,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="10">
@@ -4184,6 +4894,10 @@
       <c r="G179" s="11" t="n"/>
       <c r="H179" s="11" t="n"/>
       <c r="I179" s="11" t="n"/>
+      <c r="J179" s="11">
+        <f>IF(B179="","",IFERROR(RIGHT(B179,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B179,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="10">
@@ -4198,6 +4912,10 @@
       <c r="G180" s="11" t="n"/>
       <c r="H180" s="11" t="n"/>
       <c r="I180" s="11" t="n"/>
+      <c r="J180" s="11">
+        <f>IF(B180="","",IFERROR(RIGHT(B180,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B180,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="10">
@@ -4212,6 +4930,10 @@
       <c r="G181" s="11" t="n"/>
       <c r="H181" s="11" t="n"/>
       <c r="I181" s="11" t="n"/>
+      <c r="J181" s="11">
+        <f>IF(B181="","",IFERROR(RIGHT(B181,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B181,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="10">
@@ -4226,6 +4948,10 @@
       <c r="G182" s="11" t="n"/>
       <c r="H182" s="11" t="n"/>
       <c r="I182" s="11" t="n"/>
+      <c r="J182" s="11">
+        <f>IF(B182="","",IFERROR(RIGHT(B182,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B182,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="10">
@@ -4240,6 +4966,10 @@
       <c r="G183" s="11" t="n"/>
       <c r="H183" s="11" t="n"/>
       <c r="I183" s="11" t="n"/>
+      <c r="J183" s="11">
+        <f>IF(B183="","",IFERROR(RIGHT(B183,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B183,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="10">
@@ -4254,6 +4984,10 @@
       <c r="G184" s="11" t="n"/>
       <c r="H184" s="11" t="n"/>
       <c r="I184" s="11" t="n"/>
+      <c r="J184" s="11">
+        <f>IF(B184="","",IFERROR(RIGHT(B184,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B184,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="10">
@@ -4268,6 +5002,10 @@
       <c r="G185" s="11" t="n"/>
       <c r="H185" s="11" t="n"/>
       <c r="I185" s="11" t="n"/>
+      <c r="J185" s="11">
+        <f>IF(B185="","",IFERROR(RIGHT(B185,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B185,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="10">
@@ -4282,6 +5020,10 @@
       <c r="G186" s="11" t="n"/>
       <c r="H186" s="11" t="n"/>
       <c r="I186" s="11" t="n"/>
+      <c r="J186" s="11">
+        <f>IF(B186="","",IFERROR(RIGHT(B186,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B186,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="10">
@@ -4296,6 +5038,10 @@
       <c r="G187" s="11" t="n"/>
       <c r="H187" s="11" t="n"/>
       <c r="I187" s="11" t="n"/>
+      <c r="J187" s="11">
+        <f>IF(B187="","",IFERROR(RIGHT(B187,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B187,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="10">
@@ -4310,6 +5056,10 @@
       <c r="G188" s="11" t="n"/>
       <c r="H188" s="11" t="n"/>
       <c r="I188" s="11" t="n"/>
+      <c r="J188" s="11">
+        <f>IF(B188="","",IFERROR(RIGHT(B188,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B188,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="10">
@@ -4324,6 +5074,10 @@
       <c r="G189" s="11" t="n"/>
       <c r="H189" s="11" t="n"/>
       <c r="I189" s="11" t="n"/>
+      <c r="J189" s="11">
+        <f>IF(B189="","",IFERROR(RIGHT(B189,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B189,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="10">
@@ -4338,6 +5092,10 @@
       <c r="G190" s="11" t="n"/>
       <c r="H190" s="11" t="n"/>
       <c r="I190" s="11" t="n"/>
+      <c r="J190" s="11">
+        <f>IF(B190="","",IFERROR(RIGHT(B190,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B190,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="10">
@@ -4352,6 +5110,10 @@
       <c r="G191" s="11" t="n"/>
       <c r="H191" s="11" t="n"/>
       <c r="I191" s="11" t="n"/>
+      <c r="J191" s="11">
+        <f>IF(B191="","",IFERROR(RIGHT(B191,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B191,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="10">
@@ -4366,6 +5128,10 @@
       <c r="G192" s="11" t="n"/>
       <c r="H192" s="11" t="n"/>
       <c r="I192" s="11" t="n"/>
+      <c r="J192" s="11">
+        <f>IF(B192="","",IFERROR(RIGHT(B192,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B192,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="10">
@@ -4380,6 +5146,10 @@
       <c r="G193" s="11" t="n"/>
       <c r="H193" s="11" t="n"/>
       <c r="I193" s="11" t="n"/>
+      <c r="J193" s="11">
+        <f>IF(B193="","",IFERROR(RIGHT(B193,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B193,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="10">
@@ -4394,6 +5164,10 @@
       <c r="G194" s="11" t="n"/>
       <c r="H194" s="11" t="n"/>
       <c r="I194" s="11" t="n"/>
+      <c r="J194" s="11">
+        <f>IF(B194="","",IFERROR(RIGHT(B194,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B194,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="10">
@@ -4408,6 +5182,10 @@
       <c r="G195" s="11" t="n"/>
       <c r="H195" s="11" t="n"/>
       <c r="I195" s="11" t="n"/>
+      <c r="J195" s="11">
+        <f>IF(B195="","",IFERROR(RIGHT(B195,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B195,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="10">
@@ -4422,6 +5200,10 @@
       <c r="G196" s="11" t="n"/>
       <c r="H196" s="11" t="n"/>
       <c r="I196" s="11" t="n"/>
+      <c r="J196" s="11">
+        <f>IF(B196="","",IFERROR(RIGHT(B196,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B196,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="10">
@@ -4436,6 +5218,10 @@
       <c r="G197" s="11" t="n"/>
       <c r="H197" s="11" t="n"/>
       <c r="I197" s="11" t="n"/>
+      <c r="J197" s="11">
+        <f>IF(B197="","",IFERROR(RIGHT(B197,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B197,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="10">
@@ -4450,6 +5236,10 @@
       <c r="G198" s="11" t="n"/>
       <c r="H198" s="11" t="n"/>
       <c r="I198" s="11" t="n"/>
+      <c r="J198" s="11">
+        <f>IF(B198="","",IFERROR(RIGHT(B198,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B198,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="10">
@@ -4464,6 +5254,10 @@
       <c r="G199" s="11" t="n"/>
       <c r="H199" s="11" t="n"/>
       <c r="I199" s="11" t="n"/>
+      <c r="J199" s="11">
+        <f>IF(B199="","",IFERROR(RIGHT(B199,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B199,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="10">
@@ -4478,6 +5272,10 @@
       <c r="G200" s="11" t="n"/>
       <c r="H200" s="11" t="n"/>
       <c r="I200" s="11" t="n"/>
+      <c r="J200" s="11">
+        <f>IF(B200="","",IFERROR(RIGHT(B200,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B200,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="10">
@@ -4492,6 +5290,10 @@
       <c r="G201" s="11" t="n"/>
       <c r="H201" s="11" t="n"/>
       <c r="I201" s="11" t="n"/>
+      <c r="J201" s="11">
+        <f>IF(B201="","",IFERROR(RIGHT(B201,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B201,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="10">
@@ -4506,6 +5308,10 @@
       <c r="G202" s="11" t="n"/>
       <c r="H202" s="11" t="n"/>
       <c r="I202" s="11" t="n"/>
+      <c r="J202" s="11">
+        <f>IF(B202="","",IFERROR(RIGHT(B202,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B202,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="10">
@@ -4520,6 +5326,10 @@
       <c r="G203" s="11" t="n"/>
       <c r="H203" s="11" t="n"/>
       <c r="I203" s="11" t="n"/>
+      <c r="J203" s="11">
+        <f>IF(B203="","",IFERROR(RIGHT(B203,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B203,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="10">
@@ -4534,6 +5344,10 @@
       <c r="G204" s="11" t="n"/>
       <c r="H204" s="11" t="n"/>
       <c r="I204" s="11" t="n"/>
+      <c r="J204" s="11">
+        <f>IF(B204="","",IFERROR(RIGHT(B204,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B204,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="10">
@@ -4548,6 +5362,10 @@
       <c r="G205" s="11" t="n"/>
       <c r="H205" s="11" t="n"/>
       <c r="I205" s="11" t="n"/>
+      <c r="J205" s="11">
+        <f>IF(B205="","",IFERROR(RIGHT(B205,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B205,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="10">
@@ -4562,6 +5380,10 @@
       <c r="G206" s="11" t="n"/>
       <c r="H206" s="11" t="n"/>
       <c r="I206" s="11" t="n"/>
+      <c r="J206" s="11">
+        <f>IF(B206="","",IFERROR(RIGHT(B206,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B206,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="10">
@@ -4576,6 +5398,10 @@
       <c r="G207" s="11" t="n"/>
       <c r="H207" s="11" t="n"/>
       <c r="I207" s="11" t="n"/>
+      <c r="J207" s="11">
+        <f>IF(B207="","",IFERROR(RIGHT(B207,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B207,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="10">
@@ -4590,6 +5416,10 @@
       <c r="G208" s="11" t="n"/>
       <c r="H208" s="11" t="n"/>
       <c r="I208" s="11" t="n"/>
+      <c r="J208" s="11">
+        <f>IF(B208="","",IFERROR(RIGHT(B208,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B208,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="10">
@@ -4604,6 +5434,10 @@
       <c r="G209" s="11" t="n"/>
       <c r="H209" s="11" t="n"/>
       <c r="I209" s="11" t="n"/>
+      <c r="J209" s="11">
+        <f>IF(B209="","",IFERROR(RIGHT(B209,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B209,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="10">
@@ -4618,6 +5452,10 @@
       <c r="G210" s="11" t="n"/>
       <c r="H210" s="11" t="n"/>
       <c r="I210" s="11" t="n"/>
+      <c r="J210" s="11">
+        <f>IF(B210="","",IFERROR(RIGHT(B210,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B210,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="10">
@@ -4632,6 +5470,10 @@
       <c r="G211" s="11" t="n"/>
       <c r="H211" s="11" t="n"/>
       <c r="I211" s="11" t="n"/>
+      <c r="J211" s="11">
+        <f>IF(B211="","",IFERROR(RIGHT(B211,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B211,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="10">
@@ -4646,6 +5488,10 @@
       <c r="G212" s="11" t="n"/>
       <c r="H212" s="11" t="n"/>
       <c r="I212" s="11" t="n"/>
+      <c r="J212" s="11">
+        <f>IF(B212="","",IFERROR(RIGHT(B212,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B212,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="10">
@@ -4660,6 +5506,10 @@
       <c r="G213" s="11" t="n"/>
       <c r="H213" s="11" t="n"/>
       <c r="I213" s="11" t="n"/>
+      <c r="J213" s="11">
+        <f>IF(B213="","",IFERROR(RIGHT(B213,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B213,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="10">
@@ -4674,6 +5524,10 @@
       <c r="G214" s="11" t="n"/>
       <c r="H214" s="11" t="n"/>
       <c r="I214" s="11" t="n"/>
+      <c r="J214" s="11">
+        <f>IF(B214="","",IFERROR(RIGHT(B214,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B214,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="10">
@@ -4688,6 +5542,10 @@
       <c r="G215" s="11" t="n"/>
       <c r="H215" s="11" t="n"/>
       <c r="I215" s="11" t="n"/>
+      <c r="J215" s="11">
+        <f>IF(B215="","",IFERROR(RIGHT(B215,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B215,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="10">
@@ -4702,6 +5560,10 @@
       <c r="G216" s="11" t="n"/>
       <c r="H216" s="11" t="n"/>
       <c r="I216" s="11" t="n"/>
+      <c r="J216" s="11">
+        <f>IF(B216="","",IFERROR(RIGHT(B216,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B216,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="10">
@@ -4716,6 +5578,10 @@
       <c r="G217" s="11" t="n"/>
       <c r="H217" s="11" t="n"/>
       <c r="I217" s="11" t="n"/>
+      <c r="J217" s="11">
+        <f>IF(B217="","",IFERROR(RIGHT(B217,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B217,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="10">
@@ -4730,6 +5596,10 @@
       <c r="G218" s="11" t="n"/>
       <c r="H218" s="11" t="n"/>
       <c r="I218" s="11" t="n"/>
+      <c r="J218" s="11">
+        <f>IF(B218="","",IFERROR(RIGHT(B218,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B218,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="10">
@@ -4744,6 +5614,10 @@
       <c r="G219" s="11" t="n"/>
       <c r="H219" s="11" t="n"/>
       <c r="I219" s="11" t="n"/>
+      <c r="J219" s="11">
+        <f>IF(B219="","",IFERROR(RIGHT(B219,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B219,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="10">
@@ -4758,6 +5632,10 @@
       <c r="G220" s="11" t="n"/>
       <c r="H220" s="11" t="n"/>
       <c r="I220" s="11" t="n"/>
+      <c r="J220" s="11">
+        <f>IF(B220="","",IFERROR(RIGHT(B220,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B220,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="10">
@@ -4772,6 +5650,10 @@
       <c r="G221" s="11" t="n"/>
       <c r="H221" s="11" t="n"/>
       <c r="I221" s="11" t="n"/>
+      <c r="J221" s="11">
+        <f>IF(B221="","",IFERROR(RIGHT(B221,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B221,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="10">
@@ -4786,6 +5668,10 @@
       <c r="G222" s="11" t="n"/>
       <c r="H222" s="11" t="n"/>
       <c r="I222" s="11" t="n"/>
+      <c r="J222" s="11">
+        <f>IF(B222="","",IFERROR(RIGHT(B222,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B222,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="10">
@@ -4800,6 +5686,10 @@
       <c r="G223" s="11" t="n"/>
       <c r="H223" s="11" t="n"/>
       <c r="I223" s="11" t="n"/>
+      <c r="J223" s="11">
+        <f>IF(B223="","",IFERROR(RIGHT(B223,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B223,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="10">
@@ -4814,6 +5704,10 @@
       <c r="G224" s="11" t="n"/>
       <c r="H224" s="11" t="n"/>
       <c r="I224" s="11" t="n"/>
+      <c r="J224" s="11">
+        <f>IF(B224="","",IFERROR(RIGHT(B224,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B224,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="10">
@@ -4828,6 +5722,10 @@
       <c r="G225" s="11" t="n"/>
       <c r="H225" s="11" t="n"/>
       <c r="I225" s="11" t="n"/>
+      <c r="J225" s="11">
+        <f>IF(B225="","",IFERROR(RIGHT(B225,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B225,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="10">
@@ -4842,6 +5740,10 @@
       <c r="G226" s="11" t="n"/>
       <c r="H226" s="11" t="n"/>
       <c r="I226" s="11" t="n"/>
+      <c r="J226" s="11">
+        <f>IF(B226="","",IFERROR(RIGHT(B226,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B226,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="10">
@@ -4856,6 +5758,10 @@
       <c r="G227" s="11" t="n"/>
       <c r="H227" s="11" t="n"/>
       <c r="I227" s="11" t="n"/>
+      <c r="J227" s="11">
+        <f>IF(B227="","",IFERROR(RIGHT(B227,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B227,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="10">
@@ -4870,6 +5776,10 @@
       <c r="G228" s="11" t="n"/>
       <c r="H228" s="11" t="n"/>
       <c r="I228" s="11" t="n"/>
+      <c r="J228" s="11">
+        <f>IF(B228="","",IFERROR(RIGHT(B228,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B228,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="10">
@@ -4884,6 +5794,10 @@
       <c r="G229" s="11" t="n"/>
       <c r="H229" s="11" t="n"/>
       <c r="I229" s="11" t="n"/>
+      <c r="J229" s="11">
+        <f>IF(B229="","",IFERROR(RIGHT(B229,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B229,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="10">
@@ -4898,6 +5812,10 @@
       <c r="G230" s="11" t="n"/>
       <c r="H230" s="11" t="n"/>
       <c r="I230" s="11" t="n"/>
+      <c r="J230" s="11">
+        <f>IF(B230="","",IFERROR(RIGHT(B230,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B230,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="10">
@@ -4912,6 +5830,10 @@
       <c r="G231" s="11" t="n"/>
       <c r="H231" s="11" t="n"/>
       <c r="I231" s="11" t="n"/>
+      <c r="J231" s="11">
+        <f>IF(B231="","",IFERROR(RIGHT(B231,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B231,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="10">
@@ -4926,6 +5848,10 @@
       <c r="G232" s="11" t="n"/>
       <c r="H232" s="11" t="n"/>
       <c r="I232" s="11" t="n"/>
+      <c r="J232" s="11">
+        <f>IF(B232="","",IFERROR(RIGHT(B232,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B232,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="10">
@@ -4940,6 +5866,10 @@
       <c r="G233" s="11" t="n"/>
       <c r="H233" s="11" t="n"/>
       <c r="I233" s="11" t="n"/>
+      <c r="J233" s="11">
+        <f>IF(B233="","",IFERROR(RIGHT(B233,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B233,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="10">
@@ -4954,6 +5884,10 @@
       <c r="G234" s="11" t="n"/>
       <c r="H234" s="11" t="n"/>
       <c r="I234" s="11" t="n"/>
+      <c r="J234" s="11">
+        <f>IF(B234="","",IFERROR(RIGHT(B234,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B234,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="10">
@@ -4968,6 +5902,10 @@
       <c r="G235" s="11" t="n"/>
       <c r="H235" s="11" t="n"/>
       <c r="I235" s="11" t="n"/>
+      <c r="J235" s="11">
+        <f>IF(B235="","",IFERROR(RIGHT(B235,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B235,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="10">
@@ -4982,6 +5920,10 @@
       <c r="G236" s="11" t="n"/>
       <c r="H236" s="11" t="n"/>
       <c r="I236" s="11" t="n"/>
+      <c r="J236" s="11">
+        <f>IF(B236="","",IFERROR(RIGHT(B236,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B236,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="10">
@@ -4996,6 +5938,10 @@
       <c r="G237" s="11" t="n"/>
       <c r="H237" s="11" t="n"/>
       <c r="I237" s="11" t="n"/>
+      <c r="J237" s="11">
+        <f>IF(B237="","",IFERROR(RIGHT(B237,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B237,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="10">
@@ -5010,6 +5956,10 @@
       <c r="G238" s="11" t="n"/>
       <c r="H238" s="11" t="n"/>
       <c r="I238" s="11" t="n"/>
+      <c r="J238" s="11">
+        <f>IF(B238="","",IFERROR(RIGHT(B238,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B238,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="10">
@@ -5024,6 +5974,10 @@
       <c r="G239" s="11" t="n"/>
       <c r="H239" s="11" t="n"/>
       <c r="I239" s="11" t="n"/>
+      <c r="J239" s="11">
+        <f>IF(B239="","",IFERROR(RIGHT(B239,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B239,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="10">
@@ -5038,6 +5992,10 @@
       <c r="G240" s="11" t="n"/>
       <c r="H240" s="11" t="n"/>
       <c r="I240" s="11" t="n"/>
+      <c r="J240" s="11">
+        <f>IF(B240="","",IFERROR(RIGHT(B240,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B240,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="10">
@@ -5052,6 +6010,10 @@
       <c r="G241" s="11" t="n"/>
       <c r="H241" s="11" t="n"/>
       <c r="I241" s="11" t="n"/>
+      <c r="J241" s="11">
+        <f>IF(B241="","",IFERROR(RIGHT(B241,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B241,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="10">
@@ -5066,6 +6028,10 @@
       <c r="G242" s="11" t="n"/>
       <c r="H242" s="11" t="n"/>
       <c r="I242" s="11" t="n"/>
+      <c r="J242" s="11">
+        <f>IF(B242="","",IFERROR(RIGHT(B242,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B242,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="10">
@@ -5080,6 +6046,10 @@
       <c r="G243" s="11" t="n"/>
       <c r="H243" s="11" t="n"/>
       <c r="I243" s="11" t="n"/>
+      <c r="J243" s="11">
+        <f>IF(B243="","",IFERROR(RIGHT(B243,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B243,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="10">
@@ -5094,6 +6064,10 @@
       <c r="G244" s="11" t="n"/>
       <c r="H244" s="11" t="n"/>
       <c r="I244" s="11" t="n"/>
+      <c r="J244" s="11">
+        <f>IF(B244="","",IFERROR(RIGHT(B244,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B244,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="10">
@@ -5108,6 +6082,10 @@
       <c r="G245" s="11" t="n"/>
       <c r="H245" s="11" t="n"/>
       <c r="I245" s="11" t="n"/>
+      <c r="J245" s="11">
+        <f>IF(B245="","",IFERROR(RIGHT(B245,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B245,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="10">
@@ -5122,6 +6100,10 @@
       <c r="G246" s="11" t="n"/>
       <c r="H246" s="11" t="n"/>
       <c r="I246" s="11" t="n"/>
+      <c r="J246" s="11">
+        <f>IF(B246="","",IFERROR(RIGHT(B246,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B246,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="10">
@@ -5136,6 +6118,10 @@
       <c r="G247" s="11" t="n"/>
       <c r="H247" s="11" t="n"/>
       <c r="I247" s="11" t="n"/>
+      <c r="J247" s="11">
+        <f>IF(B247="","",IFERROR(RIGHT(B247,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B247,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="10">
@@ -5150,6 +6136,10 @@
       <c r="G248" s="11" t="n"/>
       <c r="H248" s="11" t="n"/>
       <c r="I248" s="11" t="n"/>
+      <c r="J248" s="11">
+        <f>IF(B248="","",IFERROR(RIGHT(B248,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B248,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="10">
@@ -5164,6 +6154,10 @@
       <c r="G249" s="11" t="n"/>
       <c r="H249" s="11" t="n"/>
       <c r="I249" s="11" t="n"/>
+      <c r="J249" s="11">
+        <f>IF(B249="","",IFERROR(RIGHT(B249,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B249,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="10">
@@ -5178,6 +6172,10 @@
       <c r="G250" s="11" t="n"/>
       <c r="H250" s="11" t="n"/>
       <c r="I250" s="11" t="n"/>
+      <c r="J250" s="11">
+        <f>IF(B250="","",IFERROR(RIGHT(B250,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B250,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="10">
@@ -5192,6 +6190,10 @@
       <c r="G251" s="11" t="n"/>
       <c r="H251" s="11" t="n"/>
       <c r="I251" s="11" t="n"/>
+      <c r="J251" s="11">
+        <f>IF(B251="","",IFERROR(RIGHT(B251,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B251,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="10">
@@ -5206,6 +6208,10 @@
       <c r="G252" s="11" t="n"/>
       <c r="H252" s="11" t="n"/>
       <c r="I252" s="11" t="n"/>
+      <c r="J252" s="11">
+        <f>IF(B252="","",IFERROR(RIGHT(B252,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B252,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="10">
@@ -5220,6 +6226,10 @@
       <c r="G253" s="11" t="n"/>
       <c r="H253" s="11" t="n"/>
       <c r="I253" s="11" t="n"/>
+      <c r="J253" s="11">
+        <f>IF(B253="","",IFERROR(RIGHT(B253,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B253,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="10">
@@ -5234,6 +6244,10 @@
       <c r="G254" s="11" t="n"/>
       <c r="H254" s="11" t="n"/>
       <c r="I254" s="11" t="n"/>
+      <c r="J254" s="11">
+        <f>IF(B254="","",IFERROR(RIGHT(B254,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B254,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="10">
@@ -5248,6 +6262,10 @@
       <c r="G255" s="11" t="n"/>
       <c r="H255" s="11" t="n"/>
       <c r="I255" s="11" t="n"/>
+      <c r="J255" s="11">
+        <f>IF(B255="","",IFERROR(RIGHT(B255,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B255,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="10">
@@ -5262,6 +6280,10 @@
       <c r="G256" s="11" t="n"/>
       <c r="H256" s="11" t="n"/>
       <c r="I256" s="11" t="n"/>
+      <c r="J256" s="11">
+        <f>IF(B256="","",IFERROR(RIGHT(B256,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B256,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="10">
@@ -5276,6 +6298,10 @@
       <c r="G257" s="11" t="n"/>
       <c r="H257" s="11" t="n"/>
       <c r="I257" s="11" t="n"/>
+      <c r="J257" s="11">
+        <f>IF(B257="","",IFERROR(RIGHT(B257,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B257,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="10">
@@ -5290,6 +6316,10 @@
       <c r="G258" s="11" t="n"/>
       <c r="H258" s="11" t="n"/>
       <c r="I258" s="11" t="n"/>
+      <c r="J258" s="11">
+        <f>IF(B258="","",IFERROR(RIGHT(B258,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B258,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="10">
@@ -5304,6 +6334,10 @@
       <c r="G259" s="11" t="n"/>
       <c r="H259" s="11" t="n"/>
       <c r="I259" s="11" t="n"/>
+      <c r="J259" s="11">
+        <f>IF(B259="","",IFERROR(RIGHT(B259,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B259,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="10">
@@ -5318,6 +6352,10 @@
       <c r="G260" s="11" t="n"/>
       <c r="H260" s="11" t="n"/>
       <c r="I260" s="11" t="n"/>
+      <c r="J260" s="11">
+        <f>IF(B260="","",IFERROR(RIGHT(B260,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B260,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="10">
@@ -5332,6 +6370,10 @@
       <c r="G261" s="11" t="n"/>
       <c r="H261" s="11" t="n"/>
       <c r="I261" s="11" t="n"/>
+      <c r="J261" s="11">
+        <f>IF(B261="","",IFERROR(RIGHT(B261,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B261,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="10">
@@ -5346,6 +6388,10 @@
       <c r="G262" s="11" t="n"/>
       <c r="H262" s="11" t="n"/>
       <c r="I262" s="11" t="n"/>
+      <c r="J262" s="11">
+        <f>IF(B262="","",IFERROR(RIGHT(B262,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B262,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="10">
@@ -5360,6 +6406,10 @@
       <c r="G263" s="11" t="n"/>
       <c r="H263" s="11" t="n"/>
       <c r="I263" s="11" t="n"/>
+      <c r="J263" s="11">
+        <f>IF(B263="","",IFERROR(RIGHT(B263,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B263,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="10">
@@ -5374,6 +6424,10 @@
       <c r="G264" s="11" t="n"/>
       <c r="H264" s="11" t="n"/>
       <c r="I264" s="11" t="n"/>
+      <c r="J264" s="11">
+        <f>IF(B264="","",IFERROR(RIGHT(B264,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B264,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="10">
@@ -5388,6 +6442,10 @@
       <c r="G265" s="11" t="n"/>
       <c r="H265" s="11" t="n"/>
       <c r="I265" s="11" t="n"/>
+      <c r="J265" s="11">
+        <f>IF(B265="","",IFERROR(RIGHT(B265,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B265,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="10">
@@ -5402,6 +6460,10 @@
       <c r="G266" s="11" t="n"/>
       <c r="H266" s="11" t="n"/>
       <c r="I266" s="11" t="n"/>
+      <c r="J266" s="11">
+        <f>IF(B266="","",IFERROR(RIGHT(B266,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B266,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="10">
@@ -5416,6 +6478,10 @@
       <c r="G267" s="11" t="n"/>
       <c r="H267" s="11" t="n"/>
       <c r="I267" s="11" t="n"/>
+      <c r="J267" s="11">
+        <f>IF(B267="","",IFERROR(RIGHT(B267,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B267,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="10">
@@ -5430,6 +6496,10 @@
       <c r="G268" s="11" t="n"/>
       <c r="H268" s="11" t="n"/>
       <c r="I268" s="11" t="n"/>
+      <c r="J268" s="11">
+        <f>IF(B268="","",IFERROR(RIGHT(B268,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B268,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="10">
@@ -5444,6 +6514,10 @@
       <c r="G269" s="11" t="n"/>
       <c r="H269" s="11" t="n"/>
       <c r="I269" s="11" t="n"/>
+      <c r="J269" s="11">
+        <f>IF(B269="","",IFERROR(RIGHT(B269,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B269,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="10">
@@ -5458,6 +6532,10 @@
       <c r="G270" s="11" t="n"/>
       <c r="H270" s="11" t="n"/>
       <c r="I270" s="11" t="n"/>
+      <c r="J270" s="11">
+        <f>IF(B270="","",IFERROR(RIGHT(B270,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B270,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="10">
@@ -5472,6 +6550,10 @@
       <c r="G271" s="11" t="n"/>
       <c r="H271" s="11" t="n"/>
       <c r="I271" s="11" t="n"/>
+      <c r="J271" s="11">
+        <f>IF(B271="","",IFERROR(RIGHT(B271,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B271,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="10">
@@ -5486,6 +6568,10 @@
       <c r="G272" s="11" t="n"/>
       <c r="H272" s="11" t="n"/>
       <c r="I272" s="11" t="n"/>
+      <c r="J272" s="11">
+        <f>IF(B272="","",IFERROR(RIGHT(B272,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B272,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="10">
@@ -5500,6 +6586,10 @@
       <c r="G273" s="11" t="n"/>
       <c r="H273" s="11" t="n"/>
       <c r="I273" s="11" t="n"/>
+      <c r="J273" s="11">
+        <f>IF(B273="","",IFERROR(RIGHT(B273,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B273,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="10">
@@ -5514,6 +6604,10 @@
       <c r="G274" s="11" t="n"/>
       <c r="H274" s="11" t="n"/>
       <c r="I274" s="11" t="n"/>
+      <c r="J274" s="11">
+        <f>IF(B274="","",IFERROR(RIGHT(B274,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B274,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="10">
@@ -5528,6 +6622,10 @@
       <c r="G275" s="11" t="n"/>
       <c r="H275" s="11" t="n"/>
       <c r="I275" s="11" t="n"/>
+      <c r="J275" s="11">
+        <f>IF(B275="","",IFERROR(RIGHT(B275,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B275,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="10">
@@ -5542,6 +6640,10 @@
       <c r="G276" s="11" t="n"/>
       <c r="H276" s="11" t="n"/>
       <c r="I276" s="11" t="n"/>
+      <c r="J276" s="11">
+        <f>IF(B276="","",IFERROR(RIGHT(B276,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B276,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="10">
@@ -5556,6 +6658,10 @@
       <c r="G277" s="11" t="n"/>
       <c r="H277" s="11" t="n"/>
       <c r="I277" s="11" t="n"/>
+      <c r="J277" s="11">
+        <f>IF(B277="","",IFERROR(RIGHT(B277,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B277,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="10">
@@ -5570,6 +6676,10 @@
       <c r="G278" s="11" t="n"/>
       <c r="H278" s="11" t="n"/>
       <c r="I278" s="11" t="n"/>
+      <c r="J278" s="11">
+        <f>IF(B278="","",IFERROR(RIGHT(B278,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B278,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="10">
@@ -5584,6 +6694,10 @@
       <c r="G279" s="11" t="n"/>
       <c r="H279" s="11" t="n"/>
       <c r="I279" s="11" t="n"/>
+      <c r="J279" s="11">
+        <f>IF(B279="","",IFERROR(RIGHT(B279,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B279,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="10">
@@ -5598,6 +6712,10 @@
       <c r="G280" s="11" t="n"/>
       <c r="H280" s="11" t="n"/>
       <c r="I280" s="11" t="n"/>
+      <c r="J280" s="11">
+        <f>IF(B280="","",IFERROR(RIGHT(B280,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B280,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="10">
@@ -5612,6 +6730,10 @@
       <c r="G281" s="11" t="n"/>
       <c r="H281" s="11" t="n"/>
       <c r="I281" s="11" t="n"/>
+      <c r="J281" s="11">
+        <f>IF(B281="","",IFERROR(RIGHT(B281,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B281,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="10">
@@ -5626,6 +6748,10 @@
       <c r="G282" s="11" t="n"/>
       <c r="H282" s="11" t="n"/>
       <c r="I282" s="11" t="n"/>
+      <c r="J282" s="11">
+        <f>IF(B282="","",IFERROR(RIGHT(B282,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B282,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="10">
@@ -5640,6 +6766,10 @@
       <c r="G283" s="11" t="n"/>
       <c r="H283" s="11" t="n"/>
       <c r="I283" s="11" t="n"/>
+      <c r="J283" s="11">
+        <f>IF(B283="","",IFERROR(RIGHT(B283,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B283,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="10">
@@ -5654,6 +6784,10 @@
       <c r="G284" s="11" t="n"/>
       <c r="H284" s="11" t="n"/>
       <c r="I284" s="11" t="n"/>
+      <c r="J284" s="11">
+        <f>IF(B284="","",IFERROR(RIGHT(B284,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B284,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="10">
@@ -5668,6 +6802,10 @@
       <c r="G285" s="11" t="n"/>
       <c r="H285" s="11" t="n"/>
       <c r="I285" s="11" t="n"/>
+      <c r="J285" s="11">
+        <f>IF(B285="","",IFERROR(RIGHT(B285,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B285,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="10">
@@ -5682,6 +6820,10 @@
       <c r="G286" s="11" t="n"/>
       <c r="H286" s="11" t="n"/>
       <c r="I286" s="11" t="n"/>
+      <c r="J286" s="11">
+        <f>IF(B286="","",IFERROR(RIGHT(B286,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B286,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="10">
@@ -5696,6 +6838,10 @@
       <c r="G287" s="11" t="n"/>
       <c r="H287" s="11" t="n"/>
       <c r="I287" s="11" t="n"/>
+      <c r="J287" s="11">
+        <f>IF(B287="","",IFERROR(RIGHT(B287,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B287,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="10">
@@ -5710,6 +6856,10 @@
       <c r="G288" s="11" t="n"/>
       <c r="H288" s="11" t="n"/>
       <c r="I288" s="11" t="n"/>
+      <c r="J288" s="11">
+        <f>IF(B288="","",IFERROR(RIGHT(B288,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B288,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="10">
@@ -5724,6 +6874,10 @@
       <c r="G289" s="11" t="n"/>
       <c r="H289" s="11" t="n"/>
       <c r="I289" s="11" t="n"/>
+      <c r="J289" s="11">
+        <f>IF(B289="","",IFERROR(RIGHT(B289,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B289,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="10">
@@ -5738,6 +6892,10 @@
       <c r="G290" s="11" t="n"/>
       <c r="H290" s="11" t="n"/>
       <c r="I290" s="11" t="n"/>
+      <c r="J290" s="11">
+        <f>IF(B290="","",IFERROR(RIGHT(B290,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B290,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="10">
@@ -5752,6 +6910,10 @@
       <c r="G291" s="11" t="n"/>
       <c r="H291" s="11" t="n"/>
       <c r="I291" s="11" t="n"/>
+      <c r="J291" s="11">
+        <f>IF(B291="","",IFERROR(RIGHT(B291,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B291,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="10">
@@ -5766,6 +6928,10 @@
       <c r="G292" s="11" t="n"/>
       <c r="H292" s="11" t="n"/>
       <c r="I292" s="11" t="n"/>
+      <c r="J292" s="11">
+        <f>IF(B292="","",IFERROR(RIGHT(B292,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B292,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="10">
@@ -5780,6 +6946,10 @@
       <c r="G293" s="11" t="n"/>
       <c r="H293" s="11" t="n"/>
       <c r="I293" s="11" t="n"/>
+      <c r="J293" s="11">
+        <f>IF(B293="","",IFERROR(RIGHT(B293,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B293,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="10">
@@ -5794,6 +6964,10 @@
       <c r="G294" s="11" t="n"/>
       <c r="H294" s="11" t="n"/>
       <c r="I294" s="11" t="n"/>
+      <c r="J294" s="11">
+        <f>IF(B294="","",IFERROR(RIGHT(B294,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B294,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="10">
@@ -5808,6 +6982,10 @@
       <c r="G295" s="11" t="n"/>
       <c r="H295" s="11" t="n"/>
       <c r="I295" s="11" t="n"/>
+      <c r="J295" s="11">
+        <f>IF(B295="","",IFERROR(RIGHT(B295,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B295,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="10">
@@ -5822,6 +7000,10 @@
       <c r="G296" s="11" t="n"/>
       <c r="H296" s="11" t="n"/>
       <c r="I296" s="11" t="n"/>
+      <c r="J296" s="11">
+        <f>IF(B296="","",IFERROR(RIGHT(B296,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B296,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="10">
@@ -5836,6 +7018,10 @@
       <c r="G297" s="11" t="n"/>
       <c r="H297" s="11" t="n"/>
       <c r="I297" s="11" t="n"/>
+      <c r="J297" s="11">
+        <f>IF(B297="","",IFERROR(RIGHT(B297,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B297,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="10">
@@ -5850,6 +7036,10 @@
       <c r="G298" s="11" t="n"/>
       <c r="H298" s="11" t="n"/>
       <c r="I298" s="11" t="n"/>
+      <c r="J298" s="11">
+        <f>IF(B298="","",IFERROR(RIGHT(B298,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B298,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="10">
@@ -5864,6 +7054,10 @@
       <c r="G299" s="11" t="n"/>
       <c r="H299" s="11" t="n"/>
       <c r="I299" s="11" t="n"/>
+      <c r="J299" s="11">
+        <f>IF(B299="","",IFERROR(RIGHT(B299,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B299,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="10">
@@ -5878,6 +7072,10 @@
       <c r="G300" s="11" t="n"/>
       <c r="H300" s="11" t="n"/>
       <c r="I300" s="11" t="n"/>
+      <c r="J300" s="11">
+        <f>IF(B300="","",IFERROR(RIGHT(B300,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B300,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="10">
@@ -5892,6 +7090,10 @@
       <c r="G301" s="11" t="n"/>
       <c r="H301" s="11" t="n"/>
       <c r="I301" s="11" t="n"/>
+      <c r="J301" s="11">
+        <f>IF(B301="","",IFERROR(RIGHT(B301,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B301,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="10">
@@ -5906,6 +7108,10 @@
       <c r="G302" s="11" t="n"/>
       <c r="H302" s="11" t="n"/>
       <c r="I302" s="11" t="n"/>
+      <c r="J302" s="11">
+        <f>IF(B302="","",IFERROR(RIGHT(B302,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B302,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="10">
@@ -5920,6 +7126,10 @@
       <c r="G303" s="11" t="n"/>
       <c r="H303" s="11" t="n"/>
       <c r="I303" s="11" t="n"/>
+      <c r="J303" s="11">
+        <f>IF(B303="","",IFERROR(RIGHT(B303,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B303,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="10">
@@ -5934,6 +7144,10 @@
       <c r="G304" s="11" t="n"/>
       <c r="H304" s="11" t="n"/>
       <c r="I304" s="11" t="n"/>
+      <c r="J304" s="11">
+        <f>IF(B304="","",IFERROR(RIGHT(B304,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B304,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="10">
@@ -5948,6 +7162,10 @@
       <c r="G305" s="11" t="n"/>
       <c r="H305" s="11" t="n"/>
       <c r="I305" s="11" t="n"/>
+      <c r="J305" s="11">
+        <f>IF(B305="","",IFERROR(RIGHT(B305,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B305,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="10">
@@ -5962,6 +7180,10 @@
       <c r="G306" s="11" t="n"/>
       <c r="H306" s="11" t="n"/>
       <c r="I306" s="11" t="n"/>
+      <c r="J306" s="11">
+        <f>IF(B306="","",IFERROR(RIGHT(B306,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B306,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="10">
@@ -5976,6 +7198,10 @@
       <c r="G307" s="11" t="n"/>
       <c r="H307" s="11" t="n"/>
       <c r="I307" s="11" t="n"/>
+      <c r="J307" s="11">
+        <f>IF(B307="","",IFERROR(RIGHT(B307,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B307,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="10">
@@ -5990,6 +7216,10 @@
       <c r="G308" s="11" t="n"/>
       <c r="H308" s="11" t="n"/>
       <c r="I308" s="11" t="n"/>
+      <c r="J308" s="11">
+        <f>IF(B308="","",IFERROR(RIGHT(B308,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B308,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="10">
@@ -6004,6 +7234,10 @@
       <c r="G309" s="11" t="n"/>
       <c r="H309" s="11" t="n"/>
       <c r="I309" s="11" t="n"/>
+      <c r="J309" s="11">
+        <f>IF(B309="","",IFERROR(RIGHT(B309,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B309,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="10">
@@ -6018,6 +7252,10 @@
       <c r="G310" s="11" t="n"/>
       <c r="H310" s="11" t="n"/>
       <c r="I310" s="11" t="n"/>
+      <c r="J310" s="11">
+        <f>IF(B310="","",IFERROR(RIGHT(B310,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B310,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="10">
@@ -6032,9 +7270,13 @@
       <c r="G311" s="11" t="n"/>
       <c r="H311" s="11" t="n"/>
       <c r="I311" s="11" t="n"/>
+      <c r="J311" s="11">
+        <f>IF(B311="","",IFERROR(RIGHT(B311,4)&amp;" T"&amp;ROUNDUP(VALUE(MID(B311,4,2))/3,0),""))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I311"/>
+  <autoFilter ref="A5:J311"/>
   <dataValidations count="1">
     <dataValidation sqref="I6:I311" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Achat-revente,Prestation de services,Convoyage automobile"</formula1>
@@ -6045,6 +7287,637 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Chiffre d'affaires par trimestre — calculé depuis le livre des recettes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Montants encaissés, par date d'encaissement. URSSAF : 12,4 % achat-revente, 21,3 % prestations et convoyage (taux à confirmer). Livraisons Uber : URSSAF prélevée par Uber à partir de 2026 T4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Année</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Trimestre</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Période</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Déclaration avant le</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Achat-revente</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Prestation de services (Uber)</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Convoyage automobile</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Total encaissé</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>URSSAF à payer (estimation)</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>URSSAF réellement payée</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Observations</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>juillet – septembre</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>31 octobre 2026</t>
+        </is>
+      </c>
+      <c r="E5" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Achat-revente",'Livre des recettes'!$J$6:$J$311,"2026 T3")</f>
+        <v/>
+      </c>
+      <c r="F5" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Prestation de services",'Livre des recettes'!$J$6:$J$311,"2026 T3")</f>
+        <v/>
+      </c>
+      <c r="G5" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Convoyage automobile",'Livre des recettes'!$J$6:$J$311,"2026 T3")</f>
+        <v/>
+      </c>
+      <c r="H5" s="19">
+        <f>E5+F5+G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="19">
+        <f>ROUND(E5*0.124+G5*0.213+F5*0.213,2)</f>
+        <v/>
+      </c>
+      <c r="J5" s="19" t="n">
+        <v>81</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Déclaré et payé : 627 € (587 € revente + 40 € Uber).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>octobre – décembre</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>31 janvier 2027</t>
+        </is>
+      </c>
+      <c r="E6" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Achat-revente",'Livre des recettes'!$J$6:$J$311,"2026 T4")</f>
+        <v/>
+      </c>
+      <c r="F6" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Prestation de services",'Livre des recettes'!$J$6:$J$311,"2026 T4")</f>
+        <v/>
+      </c>
+      <c r="G6" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Convoyage automobile",'Livre des recettes'!$J$6:$J$311,"2026 T4")</f>
+        <v/>
+      </c>
+      <c r="H6" s="19">
+        <f>E6+F6+G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="19">
+        <f>ROUND(E6*0.124+G6*0.213,2)</f>
+        <v/>
+      </c>
+      <c r="J6" s="19" t="n"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>En cours. Ballerines Massimo Dutti (50 €) en attente du virement Vinted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B7" s="20" t="n"/>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Total 2026</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="n"/>
+      <c r="E7" s="21">
+        <f>SUM(E5:E6)</f>
+        <v/>
+      </c>
+      <c r="F7" s="21">
+        <f>SUM(F5:F6)</f>
+        <v/>
+      </c>
+      <c r="G7" s="21">
+        <f>SUM(G5:G6)</f>
+        <v/>
+      </c>
+      <c r="H7" s="21">
+        <f>SUM(H5:H6)</f>
+        <v/>
+      </c>
+      <c r="I7" s="21">
+        <f>SUM(I5:I6)</f>
+        <v/>
+      </c>
+      <c r="J7" s="21">
+        <f>SUM(J5:J6)</f>
+        <v/>
+      </c>
+      <c r="K7" s="20" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>janvier – mars</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>30 avril 2027</t>
+        </is>
+      </c>
+      <c r="E9" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Achat-revente",'Livre des recettes'!$J$6:$J$311,"2027 T1")</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Prestation de services",'Livre des recettes'!$J$6:$J$311,"2027 T1")</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Convoyage automobile",'Livre des recettes'!$J$6:$J$311,"2027 T1")</f>
+        <v/>
+      </c>
+      <c r="H9" s="19">
+        <f>E9+F9+G9</f>
+        <v/>
+      </c>
+      <c r="I9" s="19">
+        <f>ROUND(E9*0.124+G9*0.213,2)</f>
+        <v/>
+      </c>
+      <c r="J9" s="19" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>avril – juin</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>31 juillet 2027</t>
+        </is>
+      </c>
+      <c r="E10" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Achat-revente",'Livre des recettes'!$J$6:$J$311,"2027 T2")</f>
+        <v/>
+      </c>
+      <c r="F10" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Prestation de services",'Livre des recettes'!$J$6:$J$311,"2027 T2")</f>
+        <v/>
+      </c>
+      <c r="G10" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Convoyage automobile",'Livre des recettes'!$J$6:$J$311,"2027 T2")</f>
+        <v/>
+      </c>
+      <c r="H10" s="19">
+        <f>E10+F10+G10</f>
+        <v/>
+      </c>
+      <c r="I10" s="19">
+        <f>ROUND(E10*0.124+G10*0.213,2)</f>
+        <v/>
+      </c>
+      <c r="J10" s="19" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>juillet – septembre</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>31 octobre 2027</t>
+        </is>
+      </c>
+      <c r="E11" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Achat-revente",'Livre des recettes'!$J$6:$J$311,"2027 T3")</f>
+        <v/>
+      </c>
+      <c r="F11" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Prestation de services",'Livre des recettes'!$J$6:$J$311,"2027 T3")</f>
+        <v/>
+      </c>
+      <c r="G11" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Convoyage automobile",'Livre des recettes'!$J$6:$J$311,"2027 T3")</f>
+        <v/>
+      </c>
+      <c r="H11" s="19">
+        <f>E11+F11+G11</f>
+        <v/>
+      </c>
+      <c r="I11" s="19">
+        <f>ROUND(E11*0.124+G11*0.213,2)</f>
+        <v/>
+      </c>
+      <c r="J11" s="19" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>octobre – décembre</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>31 janvier 2028</t>
+        </is>
+      </c>
+      <c r="E12" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Achat-revente",'Livre des recettes'!$J$6:$J$311,"2027 T4")</f>
+        <v/>
+      </c>
+      <c r="F12" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Prestation de services",'Livre des recettes'!$J$6:$J$311,"2027 T4")</f>
+        <v/>
+      </c>
+      <c r="G12" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Convoyage automobile",'Livre des recettes'!$J$6:$J$311,"2027 T4")</f>
+        <v/>
+      </c>
+      <c r="H12" s="19">
+        <f>E12+F12+G12</f>
+        <v/>
+      </c>
+      <c r="I12" s="19">
+        <f>ROUND(E12*0.124+G12*0.213,2)</f>
+        <v/>
+      </c>
+      <c r="J12" s="19" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B13" s="20" t="n"/>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>Total 2027</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="n"/>
+      <c r="E13" s="21">
+        <f>SUM(E9:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="21">
+        <f>SUM(F9:F12)</f>
+        <v/>
+      </c>
+      <c r="G13" s="21">
+        <f>SUM(G9:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="21">
+        <f>SUM(H9:H12)</f>
+        <v/>
+      </c>
+      <c r="I13" s="21">
+        <f>SUM(I9:I12)</f>
+        <v/>
+      </c>
+      <c r="J13" s="21">
+        <f>SUM(J9:J12)</f>
+        <v/>
+      </c>
+      <c r="K13" s="20" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>janvier – mars</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>30 avril 2028</t>
+        </is>
+      </c>
+      <c r="E15" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Achat-revente",'Livre des recettes'!$J$6:$J$311,"2028 T1")</f>
+        <v/>
+      </c>
+      <c r="F15" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Prestation de services",'Livre des recettes'!$J$6:$J$311,"2028 T1")</f>
+        <v/>
+      </c>
+      <c r="G15" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Convoyage automobile",'Livre des recettes'!$J$6:$J$311,"2028 T1")</f>
+        <v/>
+      </c>
+      <c r="H15" s="19">
+        <f>E15+F15+G15</f>
+        <v/>
+      </c>
+      <c r="I15" s="19">
+        <f>ROUND(E15*0.124+G15*0.213,2)</f>
+        <v/>
+      </c>
+      <c r="J15" s="19" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>avril – juin</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>31 juillet 2028</t>
+        </is>
+      </c>
+      <c r="E16" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Achat-revente",'Livre des recettes'!$J$6:$J$311,"2028 T2")</f>
+        <v/>
+      </c>
+      <c r="F16" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Prestation de services",'Livre des recettes'!$J$6:$J$311,"2028 T2")</f>
+        <v/>
+      </c>
+      <c r="G16" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Convoyage automobile",'Livre des recettes'!$J$6:$J$311,"2028 T2")</f>
+        <v/>
+      </c>
+      <c r="H16" s="19">
+        <f>E16+F16+G16</f>
+        <v/>
+      </c>
+      <c r="I16" s="19">
+        <f>ROUND(E16*0.124+G16*0.213,2)</f>
+        <v/>
+      </c>
+      <c r="J16" s="19" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>juillet – septembre</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>31 octobre 2028</t>
+        </is>
+      </c>
+      <c r="E17" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Achat-revente",'Livre des recettes'!$J$6:$J$311,"2028 T3")</f>
+        <v/>
+      </c>
+      <c r="F17" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Prestation de services",'Livre des recettes'!$J$6:$J$311,"2028 T3")</f>
+        <v/>
+      </c>
+      <c r="G17" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Convoyage automobile",'Livre des recettes'!$J$6:$J$311,"2028 T3")</f>
+        <v/>
+      </c>
+      <c r="H17" s="19">
+        <f>E17+F17+G17</f>
+        <v/>
+      </c>
+      <c r="I17" s="19">
+        <f>ROUND(E17*0.124+G17*0.213,2)</f>
+        <v/>
+      </c>
+      <c r="J17" s="19" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>octobre – décembre</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>31 janvier 2029</t>
+        </is>
+      </c>
+      <c r="E18" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Achat-revente",'Livre des recettes'!$J$6:$J$311,"2028 T4")</f>
+        <v/>
+      </c>
+      <c r="F18" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Prestation de services",'Livre des recettes'!$J$6:$J$311,"2028 T4")</f>
+        <v/>
+      </c>
+      <c r="G18" s="19">
+        <f>SUMIFS('Livre des recettes'!$E$6:$E$311,'Livre des recettes'!$I$6:$I$311,"Convoyage automobile",'Livre des recettes'!$J$6:$J$311,"2028 T4")</f>
+        <v/>
+      </c>
+      <c r="H18" s="19">
+        <f>E18+F18+G18</f>
+        <v/>
+      </c>
+      <c r="I18" s="19">
+        <f>ROUND(E18*0.124+G18*0.213,2)</f>
+        <v/>
+      </c>
+      <c r="J18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>Total 2028</t>
+        </is>
+      </c>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="21">
+        <f>SUM(E15:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="21">
+        <f>SUM(F15:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="21">
+        <f>SUM(G15:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="21">
+        <f>SUM(H15:H18)</f>
+        <v/>
+      </c>
+      <c r="I19" s="21">
+        <f>SUM(I15:I18)</f>
+        <v/>
+      </c>
+      <c r="J19" s="21">
+        <f>SUM(J15:J18)</f>
+        <v/>
+      </c>
+      <c r="K19" s="20" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11308,7 +13181,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Convoyage Hiflow : seule la prestation (67 €) est inscrite, frais de 94,80 € hors CA
Facture n°HIFNACIZR2026-S-3147 du 16/10/2026 : 161,80 € = 67 € de prestation
+ 94,80 € de frais remboursés (débours). Règle ajoutée au suivi comptable.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -1836,7 +1836,7 @@
         </is>
       </c>
       <c r="E16" s="12" t="n">
-        <v>161.8</v>
+        <v>67</v>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>Relevé de missions Hiflow — 4e trimestre 2026</t>
+          <t>Facture Hiflow n°HIFNACIZR2026-S-3147 du 16/10/2026 — virement 161,80 € dont 94,80 € de frais remboursés (débours, hors CA)</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Ajoute la facture Hiflow n°HIFNACIZR2026-S-3147 aux justificatifs et complète la ligne du livre des recettes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -1827,7 +1827,7 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Hiflow</t>
+          <t>Hiflow (FREECARS SAS)</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>Facture Hiflow n°HIFNACIZR2026-S-3147 du 16/10/2026 — virement 161,80 € dont 94,80 € de frais remboursés (débours, hors CA)</t>
+          <t>Facture n°HIFNACIZR2026-S-3147 du 21/10/2026 — 3 convoyages du 13 au 15/10 — virement 161,80 € dont 94,80 € de frais (hors CA)</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">

</xml_diff>